<commit_message>
Deploy: Актуализация формы 344f99aaab39c6ac95b38bccaa69c16dada0c77c
</commit_message>
<xml_diff>
--- a/docs/forms/Форма-40.xlsx
+++ b/docs/forms/Форма-40.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1129EF-C0D3-4E63-ACF7-6AA283234C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958DADD2-FA8B-4F8D-8131-F7C97016E4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="WVTMOiQwR85XTisTO4DKrfISZxNQ0BFpECcCCS000Uu+GkxcfHR6areMxt2yyc5aaThY5MfMfYqeI/nYPU05nQ==" workbookSaltValue="ribmnAY1Ux88SofCBxYDaA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -15,11 +15,16 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Форма № 40'!$A$1:$AI$60</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="180">
   <si>
     <t>1.</t>
   </si>
@@ -661,6 +666,9 @@
   </si>
   <si>
     <t>2025</t>
+  </si>
+  <si>
+    <t>2026</t>
   </si>
 </sst>
 </file>
@@ -1236,7 +1244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="175">
+  <cellXfs count="176">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1399,6 +1407,369 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1408,22 +1779,8 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -1431,34 +1788,6 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -1471,330 +1800,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -2291,43 +2300,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:60" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="150" t="s">
+      <c r="A1" s="111" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="151"/>
-      <c r="C1" s="151"/>
-      <c r="D1" s="151"/>
-      <c r="E1" s="151"/>
-      <c r="F1" s="151"/>
-      <c r="G1" s="151"/>
-      <c r="H1" s="151"/>
-      <c r="I1" s="151"/>
-      <c r="J1" s="151"/>
-      <c r="K1" s="151"/>
-      <c r="L1" s="151"/>
-      <c r="M1" s="151"/>
-      <c r="N1" s="151"/>
-      <c r="O1" s="151"/>
-      <c r="P1" s="151"/>
-      <c r="Q1" s="151"/>
-      <c r="R1" s="151"/>
-      <c r="S1" s="151"/>
-      <c r="T1" s="151"/>
-      <c r="U1" s="151"/>
-      <c r="V1" s="151"/>
-      <c r="W1" s="151"/>
-      <c r="X1" s="151"/>
-      <c r="Y1" s="151"/>
-      <c r="Z1" s="151"/>
-      <c r="AA1" s="151"/>
-      <c r="AB1" s="151"/>
-      <c r="AC1" s="151"/>
-      <c r="AD1" s="151"/>
-      <c r="AE1" s="151"/>
-      <c r="AF1" s="151"/>
-      <c r="AG1" s="151"/>
-      <c r="AH1" s="151"/>
-      <c r="AI1" s="151"/>
+      <c r="B1" s="112"/>
+      <c r="C1" s="112"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="112"/>
+      <c r="F1" s="112"/>
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="112"/>
+      <c r="L1" s="112"/>
+      <c r="M1" s="112"/>
+      <c r="N1" s="112"/>
+      <c r="O1" s="112"/>
+      <c r="P1" s="112"/>
+      <c r="Q1" s="112"/>
+      <c r="R1" s="112"/>
+      <c r="S1" s="112"/>
+      <c r="T1" s="112"/>
+      <c r="U1" s="112"/>
+      <c r="V1" s="112"/>
+      <c r="W1" s="112"/>
+      <c r="X1" s="112"/>
+      <c r="Y1" s="112"/>
+      <c r="Z1" s="112"/>
+      <c r="AA1" s="112"/>
+      <c r="AB1" s="112"/>
+      <c r="AC1" s="112"/>
+      <c r="AD1" s="112"/>
+      <c r="AE1" s="112"/>
+      <c r="AF1" s="112"/>
+      <c r="AG1" s="112"/>
+      <c r="AH1" s="112"/>
+      <c r="AI1" s="112"/>
       <c r="AW1" s="35"/>
       <c r="AX1" s="35"/>
       <c r="AY1" s="35"/>
@@ -2491,43 +2500,43 @@
       <c r="BH4" s="35"/>
     </row>
     <row r="5" spans="1:60" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="137" t="s">
+      <c r="A5" s="134" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="137"/>
-      <c r="C5" s="137"/>
-      <c r="D5" s="137"/>
-      <c r="E5" s="137"/>
-      <c r="F5" s="137"/>
-      <c r="G5" s="137"/>
-      <c r="H5" s="137"/>
-      <c r="I5" s="137"/>
-      <c r="J5" s="137"/>
-      <c r="K5" s="137"/>
-      <c r="L5" s="137"/>
-      <c r="M5" s="137"/>
-      <c r="N5" s="137"/>
-      <c r="O5" s="137"/>
-      <c r="P5" s="137"/>
-      <c r="Q5" s="137"/>
-      <c r="R5" s="137"/>
-      <c r="S5" s="137"/>
-      <c r="T5" s="137"/>
-      <c r="U5" s="137"/>
-      <c r="V5" s="137"/>
-      <c r="W5" s="137"/>
-      <c r="X5" s="137"/>
-      <c r="Y5" s="137"/>
-      <c r="Z5" s="137"/>
-      <c r="AA5" s="137"/>
-      <c r="AB5" s="137"/>
-      <c r="AC5" s="137"/>
-      <c r="AD5" s="137"/>
-      <c r="AE5" s="137"/>
-      <c r="AF5" s="137"/>
-      <c r="AG5" s="137"/>
-      <c r="AH5" s="137"/>
-      <c r="AI5" s="137"/>
+      <c r="B5" s="134"/>
+      <c r="C5" s="134"/>
+      <c r="D5" s="134"/>
+      <c r="E5" s="134"/>
+      <c r="F5" s="134"/>
+      <c r="G5" s="134"/>
+      <c r="H5" s="134"/>
+      <c r="I5" s="134"/>
+      <c r="J5" s="134"/>
+      <c r="K5" s="134"/>
+      <c r="L5" s="134"/>
+      <c r="M5" s="134"/>
+      <c r="N5" s="134"/>
+      <c r="O5" s="134"/>
+      <c r="P5" s="134"/>
+      <c r="Q5" s="134"/>
+      <c r="R5" s="134"/>
+      <c r="S5" s="134"/>
+      <c r="T5" s="134"/>
+      <c r="U5" s="134"/>
+      <c r="V5" s="134"/>
+      <c r="W5" s="134"/>
+      <c r="X5" s="134"/>
+      <c r="Y5" s="134"/>
+      <c r="Z5" s="134"/>
+      <c r="AA5" s="134"/>
+      <c r="AB5" s="134"/>
+      <c r="AC5" s="134"/>
+      <c r="AD5" s="134"/>
+      <c r="AE5" s="134"/>
+      <c r="AF5" s="134"/>
+      <c r="AG5" s="134"/>
+      <c r="AH5" s="134"/>
+      <c r="AI5" s="134"/>
       <c r="AW5" s="35"/>
       <c r="AX5" s="35"/>
       <c r="AY5" s="35"/>
@@ -2542,41 +2551,41 @@
       <c r="BH5" s="35"/>
     </row>
     <row r="6" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="A6" s="138"/>
-      <c r="B6" s="138"/>
-      <c r="C6" s="138"/>
-      <c r="D6" s="138"/>
-      <c r="E6" s="138"/>
-      <c r="F6" s="138"/>
-      <c r="G6" s="138"/>
-      <c r="H6" s="138"/>
-      <c r="I6" s="138"/>
-      <c r="J6" s="138"/>
-      <c r="K6" s="138"/>
-      <c r="L6" s="138"/>
-      <c r="M6" s="138"/>
-      <c r="N6" s="138"/>
-      <c r="O6" s="138"/>
-      <c r="P6" s="138"/>
-      <c r="Q6" s="138"/>
-      <c r="R6" s="138"/>
-      <c r="S6" s="138"/>
-      <c r="T6" s="138"/>
-      <c r="U6" s="138"/>
-      <c r="V6" s="138"/>
-      <c r="W6" s="138"/>
-      <c r="X6" s="138"/>
-      <c r="Y6" s="138"/>
-      <c r="Z6" s="138"/>
-      <c r="AA6" s="138"/>
-      <c r="AB6" s="138"/>
-      <c r="AC6" s="138"/>
-      <c r="AD6" s="138"/>
-      <c r="AE6" s="138"/>
-      <c r="AF6" s="138"/>
-      <c r="AG6" s="138"/>
-      <c r="AH6" s="138"/>
-      <c r="AI6" s="138"/>
+      <c r="A6" s="135"/>
+      <c r="B6" s="135"/>
+      <c r="C6" s="135"/>
+      <c r="D6" s="135"/>
+      <c r="E6" s="135"/>
+      <c r="F6" s="135"/>
+      <c r="G6" s="135"/>
+      <c r="H6" s="135"/>
+      <c r="I6" s="135"/>
+      <c r="J6" s="135"/>
+      <c r="K6" s="135"/>
+      <c r="L6" s="135"/>
+      <c r="M6" s="135"/>
+      <c r="N6" s="135"/>
+      <c r="O6" s="135"/>
+      <c r="P6" s="135"/>
+      <c r="Q6" s="135"/>
+      <c r="R6" s="135"/>
+      <c r="S6" s="135"/>
+      <c r="T6" s="135"/>
+      <c r="U6" s="135"/>
+      <c r="V6" s="135"/>
+      <c r="W6" s="135"/>
+      <c r="X6" s="135"/>
+      <c r="Y6" s="135"/>
+      <c r="Z6" s="135"/>
+      <c r="AA6" s="135"/>
+      <c r="AB6" s="135"/>
+      <c r="AC6" s="135"/>
+      <c r="AD6" s="135"/>
+      <c r="AE6" s="135"/>
+      <c r="AF6" s="135"/>
+      <c r="AG6" s="135"/>
+      <c r="AH6" s="135"/>
+      <c r="AI6" s="135"/>
       <c r="AW6" s="35"/>
       <c r="AX6" s="35"/>
       <c r="AY6" s="35"/>
@@ -2594,34 +2603,34 @@
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="120" t="s">
+      <c r="B7" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="120"/>
-      <c r="D7" s="120"/>
-      <c r="E7" s="120"/>
-      <c r="F7" s="120"/>
-      <c r="G7" s="120"/>
-      <c r="H7" s="120"/>
-      <c r="I7" s="120"/>
-      <c r="J7" s="120"/>
-      <c r="K7" s="120"/>
-      <c r="L7" s="120"/>
-      <c r="M7" s="120"/>
-      <c r="N7" s="120"/>
-      <c r="O7" s="171"/>
-      <c r="P7" s="172"/>
-      <c r="Q7" s="172"/>
-      <c r="R7" s="172"/>
-      <c r="S7" s="172"/>
-      <c r="T7" s="172"/>
-      <c r="U7" s="172"/>
-      <c r="V7" s="172"/>
-      <c r="W7" s="173"/>
-      <c r="X7" s="174" t="s">
+      <c r="C7" s="74"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="74"/>
+      <c r="G7" s="74"/>
+      <c r="H7" s="74"/>
+      <c r="I7" s="74"/>
+      <c r="J7" s="74"/>
+      <c r="K7" s="74"/>
+      <c r="L7" s="74"/>
+      <c r="M7" s="74"/>
+      <c r="N7" s="74"/>
+      <c r="O7" s="61"/>
+      <c r="P7" s="62"/>
+      <c r="Q7" s="62"/>
+      <c r="R7" s="62"/>
+      <c r="S7" s="62"/>
+      <c r="T7" s="62"/>
+      <c r="U7" s="62"/>
+      <c r="V7" s="62"/>
+      <c r="W7" s="63"/>
+      <c r="X7" s="64" t="s">
         <v>169</v>
       </c>
-      <c r="Y7" s="174"/>
+      <c r="Y7" s="64"/>
       <c r="Z7" s="56"/>
       <c r="AA7" s="57"/>
       <c r="AB7" s="58"/>
@@ -2646,29 +2655,29 @@
       <c r="BH7" s="35"/>
     </row>
     <row r="8" spans="1:60" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O8" s="67" t="s">
+      <c r="O8" s="72" t="s">
         <v>170</v>
       </c>
-      <c r="P8" s="67"/>
-      <c r="Q8" s="67"/>
-      <c r="R8" s="67"/>
-      <c r="S8" s="67"/>
-      <c r="T8" s="67"/>
-      <c r="U8" s="67"/>
-      <c r="V8" s="67"/>
-      <c r="W8" s="67"/>
-      <c r="X8" s="67"/>
-      <c r="Y8" s="67"/>
-      <c r="Z8" s="67"/>
-      <c r="AA8" s="67"/>
-      <c r="AB8" s="67"/>
-      <c r="AC8" s="67"/>
-      <c r="AD8" s="67"/>
-      <c r="AE8" s="67"/>
-      <c r="AF8" s="67"/>
-      <c r="AG8" s="67"/>
-      <c r="AH8" s="67"/>
-      <c r="AI8" s="67"/>
+      <c r="P8" s="72"/>
+      <c r="Q8" s="72"/>
+      <c r="R8" s="72"/>
+      <c r="S8" s="72"/>
+      <c r="T8" s="72"/>
+      <c r="U8" s="72"/>
+      <c r="V8" s="72"/>
+      <c r="W8" s="72"/>
+      <c r="X8" s="72"/>
+      <c r="Y8" s="72"/>
+      <c r="Z8" s="72"/>
+      <c r="AA8" s="72"/>
+      <c r="AB8" s="72"/>
+      <c r="AC8" s="72"/>
+      <c r="AD8" s="72"/>
+      <c r="AE8" s="72"/>
+      <c r="AF8" s="72"/>
+      <c r="AG8" s="72"/>
+      <c r="AH8" s="72"/>
+      <c r="AI8" s="72"/>
       <c r="AW8" s="35"/>
       <c r="AX8" s="35"/>
       <c r="AY8" s="35"/>
@@ -2686,34 +2695,34 @@
       <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="118" t="s">
+      <c r="B9" s="114" t="s">
         <v>102</v>
       </c>
-      <c r="C9" s="118"/>
-      <c r="D9" s="118"/>
-      <c r="E9" s="118"/>
-      <c r="F9" s="118"/>
-      <c r="G9" s="118"/>
-      <c r="H9" s="118"/>
-      <c r="I9" s="118"/>
-      <c r="J9" s="118"/>
-      <c r="K9" s="171"/>
-      <c r="L9" s="172"/>
-      <c r="M9" s="172"/>
-      <c r="N9" s="172"/>
-      <c r="O9" s="172"/>
-      <c r="P9" s="172"/>
-      <c r="Q9" s="172"/>
-      <c r="R9" s="172"/>
-      <c r="S9" s="172"/>
-      <c r="T9" s="172"/>
-      <c r="U9" s="172"/>
-      <c r="V9" s="172"/>
-      <c r="W9" s="173"/>
-      <c r="X9" s="174" t="s">
+      <c r="C9" s="114"/>
+      <c r="D9" s="114"/>
+      <c r="E9" s="114"/>
+      <c r="F9" s="114"/>
+      <c r="G9" s="114"/>
+      <c r="H9" s="114"/>
+      <c r="I9" s="114"/>
+      <c r="J9" s="114"/>
+      <c r="K9" s="61"/>
+      <c r="L9" s="62"/>
+      <c r="M9" s="62"/>
+      <c r="N9" s="62"/>
+      <c r="O9" s="62"/>
+      <c r="P9" s="62"/>
+      <c r="Q9" s="62"/>
+      <c r="R9" s="62"/>
+      <c r="S9" s="62"/>
+      <c r="T9" s="62"/>
+      <c r="U9" s="62"/>
+      <c r="V9" s="62"/>
+      <c r="W9" s="63"/>
+      <c r="X9" s="64" t="s">
         <v>169</v>
       </c>
-      <c r="Y9" s="174"/>
+      <c r="Y9" s="64"/>
       <c r="Z9" s="56"/>
       <c r="AA9" s="57"/>
       <c r="AB9" s="58"/>
@@ -2738,34 +2747,34 @@
       <c r="BH9" s="35"/>
     </row>
     <row r="10" spans="1:60" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="J10" s="67" t="s">
+      <c r="J10" s="72" t="s">
         <v>170</v>
       </c>
-      <c r="K10" s="67"/>
-      <c r="L10" s="67"/>
-      <c r="M10" s="67"/>
-      <c r="N10" s="67"/>
-      <c r="O10" s="67"/>
-      <c r="P10" s="67"/>
-      <c r="Q10" s="67"/>
-      <c r="R10" s="67"/>
-      <c r="S10" s="67"/>
-      <c r="T10" s="67"/>
-      <c r="U10" s="67"/>
-      <c r="V10" s="67"/>
-      <c r="W10" s="67"/>
-      <c r="X10" s="67"/>
-      <c r="Y10" s="67"/>
-      <c r="Z10" s="67"/>
-      <c r="AA10" s="67"/>
-      <c r="AB10" s="67"/>
-      <c r="AC10" s="67"/>
-      <c r="AD10" s="67"/>
-      <c r="AE10" s="67"/>
-      <c r="AF10" s="67"/>
-      <c r="AG10" s="67"/>
-      <c r="AH10" s="67"/>
-      <c r="AI10" s="67"/>
+      <c r="K10" s="72"/>
+      <c r="L10" s="72"/>
+      <c r="M10" s="72"/>
+      <c r="N10" s="72"/>
+      <c r="O10" s="72"/>
+      <c r="P10" s="72"/>
+      <c r="Q10" s="72"/>
+      <c r="R10" s="72"/>
+      <c r="S10" s="72"/>
+      <c r="T10" s="72"/>
+      <c r="U10" s="72"/>
+      <c r="V10" s="72"/>
+      <c r="W10" s="72"/>
+      <c r="X10" s="72"/>
+      <c r="Y10" s="72"/>
+      <c r="Z10" s="72"/>
+      <c r="AA10" s="72"/>
+      <c r="AB10" s="72"/>
+      <c r="AC10" s="72"/>
+      <c r="AD10" s="72"/>
+      <c r="AE10" s="72"/>
+      <c r="AF10" s="72"/>
+      <c r="AG10" s="72"/>
+      <c r="AH10" s="72"/>
+      <c r="AI10" s="72"/>
       <c r="AW10" s="35"/>
       <c r="AX10" s="35"/>
       <c r="AY10" s="35"/>
@@ -2783,41 +2792,41 @@
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="140" t="s">
+      <c r="B11" s="116" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="140"/>
-      <c r="D11" s="140"/>
-      <c r="E11" s="140"/>
-      <c r="F11" s="141"/>
-      <c r="G11" s="142"/>
-      <c r="H11" s="142"/>
-      <c r="I11" s="142"/>
-      <c r="J11" s="142"/>
-      <c r="K11" s="142"/>
-      <c r="L11" s="142"/>
-      <c r="M11" s="142"/>
-      <c r="N11" s="142"/>
-      <c r="O11" s="142"/>
-      <c r="P11" s="142"/>
-      <c r="Q11" s="142"/>
-      <c r="R11" s="142"/>
-      <c r="S11" s="142"/>
-      <c r="T11" s="142"/>
-      <c r="U11" s="142"/>
-      <c r="V11" s="142"/>
-      <c r="W11" s="142"/>
-      <c r="X11" s="142"/>
-      <c r="Y11" s="142"/>
-      <c r="Z11" s="142"/>
-      <c r="AA11" s="142"/>
-      <c r="AB11" s="142"/>
-      <c r="AC11" s="142"/>
-      <c r="AD11" s="142"/>
-      <c r="AE11" s="142"/>
-      <c r="AF11" s="142"/>
-      <c r="AG11" s="142"/>
-      <c r="AH11" s="143"/>
+      <c r="C11" s="116"/>
+      <c r="D11" s="116"/>
+      <c r="E11" s="116"/>
+      <c r="F11" s="118"/>
+      <c r="G11" s="119"/>
+      <c r="H11" s="119"/>
+      <c r="I11" s="119"/>
+      <c r="J11" s="119"/>
+      <c r="K11" s="119"/>
+      <c r="L11" s="119"/>
+      <c r="M11" s="119"/>
+      <c r="N11" s="119"/>
+      <c r="O11" s="119"/>
+      <c r="P11" s="119"/>
+      <c r="Q11" s="119"/>
+      <c r="R11" s="119"/>
+      <c r="S11" s="119"/>
+      <c r="T11" s="119"/>
+      <c r="U11" s="119"/>
+      <c r="V11" s="119"/>
+      <c r="W11" s="119"/>
+      <c r="X11" s="119"/>
+      <c r="Y11" s="119"/>
+      <c r="Z11" s="119"/>
+      <c r="AA11" s="119"/>
+      <c r="AB11" s="119"/>
+      <c r="AC11" s="119"/>
+      <c r="AD11" s="119"/>
+      <c r="AE11" s="119"/>
+      <c r="AF11" s="119"/>
+      <c r="AG11" s="119"/>
+      <c r="AH11" s="120"/>
       <c r="AI11" s="14"/>
       <c r="AW11" s="35"/>
       <c r="AX11" s="35"/>
@@ -2833,38 +2842,38 @@
       <c r="BH11" s="35"/>
     </row>
     <row r="12" spans="1:60" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F12" s="67" t="s">
+      <c r="F12" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="67"/>
-      <c r="H12" s="67"/>
-      <c r="I12" s="67"/>
-      <c r="J12" s="67"/>
-      <c r="K12" s="67"/>
-      <c r="L12" s="67"/>
-      <c r="M12" s="67"/>
-      <c r="N12" s="67"/>
-      <c r="O12" s="67"/>
-      <c r="P12" s="67"/>
-      <c r="Q12" s="67"/>
-      <c r="R12" s="67"/>
-      <c r="S12" s="67"/>
-      <c r="T12" s="67"/>
-      <c r="U12" s="67"/>
-      <c r="V12" s="67"/>
-      <c r="W12" s="67"/>
-      <c r="X12" s="67"/>
-      <c r="Y12" s="67"/>
-      <c r="Z12" s="67"/>
-      <c r="AA12" s="67"/>
-      <c r="AB12" s="67"/>
-      <c r="AC12" s="67"/>
-      <c r="AD12" s="67"/>
-      <c r="AE12" s="67"/>
-      <c r="AF12" s="67"/>
-      <c r="AG12" s="67"/>
-      <c r="AH12" s="67"/>
-      <c r="AI12" s="67"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="72"/>
+      <c r="L12" s="72"/>
+      <c r="M12" s="72"/>
+      <c r="N12" s="72"/>
+      <c r="O12" s="72"/>
+      <c r="P12" s="72"/>
+      <c r="Q12" s="72"/>
+      <c r="R12" s="72"/>
+      <c r="S12" s="72"/>
+      <c r="T12" s="72"/>
+      <c r="U12" s="72"/>
+      <c r="V12" s="72"/>
+      <c r="W12" s="72"/>
+      <c r="X12" s="72"/>
+      <c r="Y12" s="72"/>
+      <c r="Z12" s="72"/>
+      <c r="AA12" s="72"/>
+      <c r="AB12" s="72"/>
+      <c r="AC12" s="72"/>
+      <c r="AD12" s="72"/>
+      <c r="AE12" s="72"/>
+      <c r="AF12" s="72"/>
+      <c r="AG12" s="72"/>
+      <c r="AH12" s="72"/>
+      <c r="AI12" s="72"/>
       <c r="AW12" s="35"/>
       <c r="AX12" s="35"/>
       <c r="AY12" s="35"/>
@@ -2879,42 +2888,42 @@
       <c r="BH12" s="35"/>
     </row>
     <row r="13" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="B13" s="118" t="s">
+      <c r="B13" s="114" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="118"/>
-      <c r="D13" s="118"/>
-      <c r="E13" s="118"/>
-      <c r="F13" s="118"/>
-      <c r="G13" s="118"/>
+      <c r="C13" s="114"/>
+      <c r="D13" s="114"/>
+      <c r="E13" s="114"/>
+      <c r="F13" s="114"/>
+      <c r="G13" s="114"/>
       <c r="H13" s="133"/>
-      <c r="I13" s="144"/>
-      <c r="J13" s="145"/>
-      <c r="K13" s="145"/>
-      <c r="L13" s="145"/>
-      <c r="M13" s="145"/>
-      <c r="N13" s="145"/>
-      <c r="O13" s="145"/>
-      <c r="P13" s="145"/>
-      <c r="Q13" s="145"/>
-      <c r="R13" s="145"/>
-      <c r="S13" s="145"/>
-      <c r="T13" s="145"/>
-      <c r="U13" s="145"/>
-      <c r="V13" s="145"/>
-      <c r="W13" s="145"/>
-      <c r="X13" s="145"/>
-      <c r="Y13" s="145"/>
-      <c r="Z13" s="145"/>
-      <c r="AA13" s="145"/>
-      <c r="AB13" s="145"/>
-      <c r="AC13" s="145"/>
-      <c r="AD13" s="145"/>
-      <c r="AE13" s="145"/>
-      <c r="AF13" s="145"/>
-      <c r="AG13" s="145"/>
-      <c r="AH13" s="145"/>
-      <c r="AI13" s="146"/>
+      <c r="I13" s="121"/>
+      <c r="J13" s="122"/>
+      <c r="K13" s="122"/>
+      <c r="L13" s="122"/>
+      <c r="M13" s="122"/>
+      <c r="N13" s="122"/>
+      <c r="O13" s="122"/>
+      <c r="P13" s="122"/>
+      <c r="Q13" s="122"/>
+      <c r="R13" s="122"/>
+      <c r="S13" s="122"/>
+      <c r="T13" s="122"/>
+      <c r="U13" s="122"/>
+      <c r="V13" s="122"/>
+      <c r="W13" s="122"/>
+      <c r="X13" s="122"/>
+      <c r="Y13" s="122"/>
+      <c r="Z13" s="122"/>
+      <c r="AA13" s="122"/>
+      <c r="AB13" s="122"/>
+      <c r="AC13" s="122"/>
+      <c r="AD13" s="122"/>
+      <c r="AE13" s="122"/>
+      <c r="AF13" s="122"/>
+      <c r="AG13" s="122"/>
+      <c r="AH13" s="122"/>
+      <c r="AI13" s="123"/>
       <c r="AW13" s="35"/>
       <c r="AX13" s="35"/>
       <c r="AY13" s="35"/>
@@ -2932,33 +2941,33 @@
       <c r="F14" s="11"/>
       <c r="G14" s="11"/>
       <c r="H14" s="11"/>
-      <c r="I14" s="147"/>
-      <c r="J14" s="148"/>
-      <c r="K14" s="148"/>
-      <c r="L14" s="148"/>
-      <c r="M14" s="148"/>
-      <c r="N14" s="148"/>
-      <c r="O14" s="148"/>
-      <c r="P14" s="148"/>
-      <c r="Q14" s="148"/>
-      <c r="R14" s="148"/>
-      <c r="S14" s="148"/>
-      <c r="T14" s="148"/>
-      <c r="U14" s="148"/>
-      <c r="V14" s="148"/>
-      <c r="W14" s="148"/>
-      <c r="X14" s="148"/>
-      <c r="Y14" s="148"/>
-      <c r="Z14" s="148"/>
-      <c r="AA14" s="148"/>
-      <c r="AB14" s="148"/>
-      <c r="AC14" s="148"/>
-      <c r="AD14" s="148"/>
-      <c r="AE14" s="148"/>
-      <c r="AF14" s="148"/>
-      <c r="AG14" s="148"/>
-      <c r="AH14" s="148"/>
-      <c r="AI14" s="149"/>
+      <c r="I14" s="124"/>
+      <c r="J14" s="125"/>
+      <c r="K14" s="125"/>
+      <c r="L14" s="125"/>
+      <c r="M14" s="125"/>
+      <c r="N14" s="125"/>
+      <c r="O14" s="125"/>
+      <c r="P14" s="125"/>
+      <c r="Q14" s="125"/>
+      <c r="R14" s="125"/>
+      <c r="S14" s="125"/>
+      <c r="T14" s="125"/>
+      <c r="U14" s="125"/>
+      <c r="V14" s="125"/>
+      <c r="W14" s="125"/>
+      <c r="X14" s="125"/>
+      <c r="Y14" s="125"/>
+      <c r="Z14" s="125"/>
+      <c r="AA14" s="125"/>
+      <c r="AB14" s="125"/>
+      <c r="AC14" s="125"/>
+      <c r="AD14" s="125"/>
+      <c r="AE14" s="125"/>
+      <c r="AF14" s="125"/>
+      <c r="AG14" s="125"/>
+      <c r="AH14" s="125"/>
+      <c r="AI14" s="126"/>
       <c r="AP14" s="38"/>
       <c r="AW14" s="35"/>
       <c r="AX14" s="35"/>
@@ -2974,35 +2983,35 @@
       <c r="BH14" s="35"/>
     </row>
     <row r="15" spans="1:60" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I15" s="95" t="s">
+      <c r="I15" s="136" t="s">
         <v>101</v>
       </c>
-      <c r="J15" s="95"/>
-      <c r="K15" s="95"/>
-      <c r="L15" s="95"/>
-      <c r="M15" s="95"/>
-      <c r="N15" s="95"/>
-      <c r="O15" s="95"/>
-      <c r="P15" s="95"/>
-      <c r="Q15" s="95"/>
-      <c r="R15" s="95"/>
-      <c r="S15" s="95"/>
-      <c r="T15" s="95"/>
-      <c r="U15" s="95"/>
-      <c r="V15" s="95"/>
-      <c r="W15" s="95"/>
-      <c r="X15" s="95"/>
-      <c r="Y15" s="95"/>
-      <c r="Z15" s="95"/>
-      <c r="AA15" s="95"/>
-      <c r="AB15" s="95"/>
-      <c r="AC15" s="95"/>
-      <c r="AD15" s="95"/>
-      <c r="AE15" s="95"/>
-      <c r="AF15" s="95"/>
-      <c r="AG15" s="95"/>
-      <c r="AH15" s="95"/>
-      <c r="AI15" s="95"/>
+      <c r="J15" s="136"/>
+      <c r="K15" s="136"/>
+      <c r="L15" s="136"/>
+      <c r="M15" s="136"/>
+      <c r="N15" s="136"/>
+      <c r="O15" s="136"/>
+      <c r="P15" s="136"/>
+      <c r="Q15" s="136"/>
+      <c r="R15" s="136"/>
+      <c r="S15" s="136"/>
+      <c r="T15" s="136"/>
+      <c r="U15" s="136"/>
+      <c r="V15" s="136"/>
+      <c r="W15" s="136"/>
+      <c r="X15" s="136"/>
+      <c r="Y15" s="136"/>
+      <c r="Z15" s="136"/>
+      <c r="AA15" s="136"/>
+      <c r="AB15" s="136"/>
+      <c r="AC15" s="136"/>
+      <c r="AD15" s="136"/>
+      <c r="AE15" s="136"/>
+      <c r="AF15" s="136"/>
+      <c r="AG15" s="136"/>
+      <c r="AH15" s="136"/>
+      <c r="AI15" s="136"/>
       <c r="AP15" s="38"/>
       <c r="AW15" s="35"/>
       <c r="AX15" s="35"/>
@@ -3021,27 +3030,28 @@
       <c r="A16" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="120" t="s">
+      <c r="B16" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="120"/>
-      <c r="D16" s="120"/>
-      <c r="E16" s="120"/>
-      <c r="F16" s="120"/>
-      <c r="G16" s="120"/>
-      <c r="H16" s="120"/>
-      <c r="I16" s="120"/>
-      <c r="J16" s="120"/>
-      <c r="K16" s="120"/>
-      <c r="L16" s="120"/>
-      <c r="M16" s="120"/>
-      <c r="N16" s="120"/>
-      <c r="O16" s="120"/>
-      <c r="P16" s="120"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="74"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="74"/>
+      <c r="K16" s="74"/>
+      <c r="L16" s="74"/>
+      <c r="M16" s="74"/>
+      <c r="N16" s="74"/>
+      <c r="O16" s="74"/>
+      <c r="P16" s="74"/>
       <c r="Q16" s="133"/>
-      <c r="R16" s="134"/>
-      <c r="S16" s="135"/>
-      <c r="T16" s="136"/>
+      <c r="R16" s="92"/>
+      <c r="S16" s="93"/>
+      <c r="T16" s="94"/>
+      <c r="AN16" s="175"/>
       <c r="AP16" s="38"/>
       <c r="AW16" s="35"/>
       <c r="AX16" s="35"/>
@@ -3057,6 +3067,7 @@
       <c r="BH16" s="35"/>
     </row>
     <row r="17" spans="1:60" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AN17" s="175"/>
       <c r="AP17" s="38"/>
       <c r="AW17" s="35"/>
       <c r="AX17" s="35"/>
@@ -3075,23 +3086,23 @@
       <c r="A18" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="120" t="s">
+      <c r="B18" s="74" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="120"/>
-      <c r="D18" s="120"/>
-      <c r="E18" s="120"/>
-      <c r="F18" s="120"/>
-      <c r="G18" s="120"/>
-      <c r="H18" s="120"/>
-      <c r="I18" s="120"/>
-      <c r="J18" s="120"/>
-      <c r="K18" s="120"/>
-      <c r="L18" s="120"/>
-      <c r="M18" s="120"/>
-      <c r="N18" s="120"/>
-      <c r="O18" s="120"/>
-      <c r="P18" s="120"/>
+      <c r="C18" s="74"/>
+      <c r="D18" s="74"/>
+      <c r="E18" s="74"/>
+      <c r="F18" s="74"/>
+      <c r="G18" s="74"/>
+      <c r="H18" s="74"/>
+      <c r="I18" s="74"/>
+      <c r="J18" s="74"/>
+      <c r="K18" s="74"/>
+      <c r="L18" s="74"/>
+      <c r="M18" s="74"/>
+      <c r="N18" s="74"/>
+      <c r="O18" s="74"/>
+      <c r="P18" s="74"/>
       <c r="Q18" s="130"/>
       <c r="R18" s="131"/>
       <c r="S18" s="131"/>
@@ -3101,20 +3112,21 @@
       <c r="W18" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="X18" s="86"/>
-      <c r="Y18" s="87"/>
-      <c r="Z18" s="88"/>
-      <c r="AA18" s="87"/>
-      <c r="AB18" s="88"/>
-      <c r="AC18" s="89"/>
+      <c r="X18" s="113"/>
+      <c r="Y18" s="69"/>
+      <c r="Z18" s="68"/>
+      <c r="AA18" s="69"/>
+      <c r="AB18" s="68"/>
+      <c r="AC18" s="70"/>
       <c r="AD18" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="AE18" s="77"/>
-      <c r="AF18" s="78"/>
-      <c r="AG18" s="78"/>
-      <c r="AH18" s="78"/>
-      <c r="AI18" s="79"/>
+      <c r="AE18" s="137"/>
+      <c r="AF18" s="138"/>
+      <c r="AG18" s="138"/>
+      <c r="AH18" s="138"/>
+      <c r="AI18" s="139"/>
+      <c r="AN18" s="175"/>
       <c r="AP18" s="38"/>
       <c r="AW18" s="35"/>
       <c r="AX18" s="35"/>
@@ -3130,52 +3142,53 @@
       <c r="BH18" s="35"/>
     </row>
     <row r="19" spans="1:60" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="67" t="s">
+      <c r="B19" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="67"/>
-      <c r="D19" s="67"/>
-      <c r="E19" s="67"/>
-      <c r="F19" s="67"/>
-      <c r="G19" s="67"/>
-      <c r="H19" s="67"/>
-      <c r="I19" s="67"/>
-      <c r="J19" s="67"/>
-      <c r="K19" s="67"/>
-      <c r="L19" s="67"/>
-      <c r="M19" s="67"/>
-      <c r="N19" s="67"/>
-      <c r="O19" s="67"/>
-      <c r="P19" s="67"/>
-      <c r="Q19" s="67" t="s">
+      <c r="C19" s="72"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
+      <c r="F19" s="72"/>
+      <c r="G19" s="72"/>
+      <c r="H19" s="72"/>
+      <c r="I19" s="72"/>
+      <c r="J19" s="72"/>
+      <c r="K19" s="72"/>
+      <c r="L19" s="72"/>
+      <c r="M19" s="72"/>
+      <c r="N19" s="72"/>
+      <c r="O19" s="72"/>
+      <c r="P19" s="72"/>
+      <c r="Q19" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="R19" s="67"/>
-      <c r="S19" s="67"/>
-      <c r="T19" s="67"/>
-      <c r="U19" s="67"/>
-      <c r="V19" s="67"/>
+      <c r="R19" s="72"/>
+      <c r="S19" s="72"/>
+      <c r="T19" s="72"/>
+      <c r="U19" s="72"/>
+      <c r="V19" s="72"/>
       <c r="W19" s="3"/>
-      <c r="X19" s="97" t="s">
+      <c r="X19" s="79" t="s">
         <v>17</v>
       </c>
-      <c r="Y19" s="97"/>
-      <c r="Z19" s="97" t="s">
+      <c r="Y19" s="79"/>
+      <c r="Z19" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="AA19" s="97"/>
-      <c r="AB19" s="97" t="s">
+      <c r="AA19" s="79"/>
+      <c r="AB19" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="AC19" s="97"/>
-      <c r="AE19" s="102" t="s">
+      <c r="AC19" s="79"/>
+      <c r="AE19" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="AF19" s="102"/>
-      <c r="AG19" s="102"/>
-      <c r="AH19" s="102"/>
-      <c r="AI19" s="102"/>
+      <c r="AF19" s="80"/>
+      <c r="AG19" s="80"/>
+      <c r="AH19" s="80"/>
+      <c r="AI19" s="80"/>
       <c r="AJ19" s="39"/>
+      <c r="AN19" s="175"/>
       <c r="AO19" s="38" t="s">
         <v>65</v>
       </c>
@@ -3208,19 +3221,19 @@
       <c r="A20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="120" t="s">
+      <c r="B20" s="74" t="s">
         <v>58</v>
       </c>
-      <c r="C20" s="120"/>
-      <c r="D20" s="120"/>
-      <c r="E20" s="120"/>
-      <c r="F20" s="120"/>
-      <c r="G20" s="120"/>
-      <c r="H20" s="120"/>
-      <c r="I20" s="120"/>
-      <c r="J20" s="120"/>
-      <c r="K20" s="120"/>
-      <c r="L20" s="120"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="74"/>
+      <c r="E20" s="74"/>
+      <c r="F20" s="74"/>
+      <c r="G20" s="74"/>
+      <c r="H20" s="74"/>
+      <c r="I20" s="74"/>
+      <c r="J20" s="74"/>
+      <c r="K20" s="74"/>
+      <c r="L20" s="74"/>
       <c r="M20" s="4"/>
       <c r="X20" s="21"/>
       <c r="Y20" s="21"/>
@@ -3228,17 +3241,18 @@
       <c r="AA20" s="21"/>
       <c r="AB20" s="21"/>
       <c r="AC20" s="21"/>
-      <c r="AE20" s="102"/>
-      <c r="AF20" s="102"/>
-      <c r="AG20" s="102"/>
-      <c r="AH20" s="102"/>
-      <c r="AI20" s="102"/>
+      <c r="AE20" s="80"/>
+      <c r="AF20" s="80"/>
+      <c r="AG20" s="80"/>
+      <c r="AH20" s="80"/>
+      <c r="AI20" s="80"/>
       <c r="AJ20" s="40" t="s">
         <v>62</v>
       </c>
       <c r="AM20" s="36" t="s">
         <v>44</v>
       </c>
+      <c r="AN20" s="175"/>
       <c r="AO20" s="38" t="s">
         <v>66</v>
       </c>
@@ -3268,53 +3282,54 @@
       <c r="BH20" s="35"/>
     </row>
     <row r="21" spans="1:60" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="139" t="s">
+      <c r="C21" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="D21" s="139"/>
-      <c r="E21" s="139"/>
-      <c r="F21" s="139"/>
-      <c r="G21" s="139"/>
-      <c r="H21" s="139"/>
-      <c r="J21" s="121" t="s">
+      <c r="D21" s="73"/>
+      <c r="E21" s="73"/>
+      <c r="F21" s="73"/>
+      <c r="G21" s="73"/>
+      <c r="H21" s="73"/>
+      <c r="J21" s="117" t="s">
         <v>77</v>
       </c>
-      <c r="K21" s="121"/>
-      <c r="L21" s="121"/>
-      <c r="M21" s="121"/>
-      <c r="N21" s="121" t="s">
+      <c r="K21" s="117"/>
+      <c r="L21" s="117"/>
+      <c r="M21" s="117"/>
+      <c r="N21" s="117" t="s">
         <v>96</v>
       </c>
-      <c r="O21" s="121"/>
-      <c r="P21" s="121"/>
-      <c r="Q21" s="121"/>
+      <c r="O21" s="117"/>
+      <c r="P21" s="117"/>
+      <c r="Q21" s="117"/>
       <c r="R21" s="23"/>
-      <c r="U21" s="139" t="s">
+      <c r="U21" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="V21" s="139"/>
-      <c r="W21" s="139"/>
-      <c r="X21" s="139"/>
-      <c r="Y21" s="139"/>
-      <c r="Z21" s="139"/>
-      <c r="AB21" s="121" t="s">
+      <c r="V21" s="73"/>
+      <c r="W21" s="73"/>
+      <c r="X21" s="73"/>
+      <c r="Y21" s="73"/>
+      <c r="Z21" s="73"/>
+      <c r="AB21" s="117" t="s">
         <v>77</v>
       </c>
-      <c r="AC21" s="121"/>
-      <c r="AD21" s="121"/>
-      <c r="AE21" s="121"/>
-      <c r="AF21" s="121" t="s">
+      <c r="AC21" s="117"/>
+      <c r="AD21" s="117"/>
+      <c r="AE21" s="117"/>
+      <c r="AF21" s="117" t="s">
         <v>96</v>
       </c>
-      <c r="AG21" s="121"/>
-      <c r="AH21" s="121"/>
-      <c r="AI21" s="121"/>
+      <c r="AG21" s="117"/>
+      <c r="AH21" s="117"/>
+      <c r="AI21" s="117"/>
       <c r="AJ21" s="39" t="s">
         <v>60</v>
       </c>
       <c r="AM21" s="36" t="s">
         <v>45</v>
       </c>
+      <c r="AN21" s="175"/>
       <c r="AO21" s="38" t="s">
         <v>67</v>
       </c>
@@ -3344,52 +3359,52 @@
       <c r="BH21" s="35"/>
     </row>
     <row r="22" spans="1:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="76" t="s">
+      <c r="A22" s="81" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="90"/>
-      <c r="C22" s="86"/>
-      <c r="D22" s="87"/>
-      <c r="E22" s="88"/>
-      <c r="F22" s="87"/>
-      <c r="G22" s="88"/>
-      <c r="H22" s="89"/>
-      <c r="I22" s="72" t="s">
+      <c r="B22" s="115"/>
+      <c r="C22" s="113"/>
+      <c r="D22" s="69"/>
+      <c r="E22" s="68"/>
+      <c r="F22" s="69"/>
+      <c r="G22" s="68"/>
+      <c r="H22" s="70"/>
+      <c r="I22" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="J22" s="73"/>
-      <c r="K22" s="74"/>
-      <c r="L22" s="74"/>
-      <c r="M22" s="75" t="s">
+      <c r="J22" s="67"/>
+      <c r="K22" s="65"/>
+      <c r="L22" s="65"/>
+      <c r="M22" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="N22" s="73"/>
-      <c r="O22" s="74"/>
-      <c r="P22" s="74"/>
+      <c r="N22" s="67"/>
+      <c r="O22" s="65"/>
+      <c r="P22" s="65"/>
       <c r="Q22" s="6"/>
       <c r="R22" s="23"/>
-      <c r="S22" s="76" t="s">
+      <c r="S22" s="81" t="s">
         <v>111</v>
       </c>
-      <c r="T22" s="90"/>
-      <c r="U22" s="86"/>
-      <c r="V22" s="87"/>
-      <c r="W22" s="88"/>
-      <c r="X22" s="87"/>
-      <c r="Y22" s="88"/>
-      <c r="Z22" s="89"/>
-      <c r="AA22" s="72" t="s">
+      <c r="T22" s="115"/>
+      <c r="U22" s="113"/>
+      <c r="V22" s="69"/>
+      <c r="W22" s="68"/>
+      <c r="X22" s="69"/>
+      <c r="Y22" s="68"/>
+      <c r="Z22" s="70"/>
+      <c r="AA22" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="AB22" s="73"/>
-      <c r="AC22" s="74"/>
-      <c r="AD22" s="74"/>
-      <c r="AE22" s="75" t="s">
+      <c r="AB22" s="67"/>
+      <c r="AC22" s="65"/>
+      <c r="AD22" s="65"/>
+      <c r="AE22" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="AF22" s="73"/>
-      <c r="AG22" s="74"/>
-      <c r="AH22" s="74"/>
+      <c r="AF22" s="67"/>
+      <c r="AG22" s="65"/>
+      <c r="AH22" s="65"/>
       <c r="AI22" s="6"/>
       <c r="AJ22" s="40" t="s">
         <v>61</v>
@@ -3400,6 +3415,7 @@
       <c r="AM22" s="36" t="s">
         <v>43</v>
       </c>
+      <c r="AN22" s="175"/>
       <c r="AO22" s="38" t="s">
         <v>68</v>
       </c>
@@ -3427,35 +3443,35 @@
       <c r="BH22" s="35"/>
     </row>
     <row r="23" spans="1:60" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="67" t="s">
+      <c r="C23" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="D23" s="67"/>
-      <c r="E23" s="67" t="s">
+      <c r="D23" s="72"/>
+      <c r="E23" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="F23" s="67"/>
-      <c r="G23" s="67" t="s">
+      <c r="F23" s="72"/>
+      <c r="G23" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="H23" s="67"/>
+      <c r="H23" s="72"/>
       <c r="L23" s="11"/>
       <c r="M23" s="5"/>
       <c r="N23" s="3"/>
       <c r="O23" s="22"/>
       <c r="R23" s="23"/>
-      <c r="U23" s="67" t="s">
+      <c r="U23" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="V23" s="67"/>
-      <c r="W23" s="67" t="s">
+      <c r="V23" s="72"/>
+      <c r="W23" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="X23" s="67"/>
-      <c r="Y23" s="67" t="s">
+      <c r="X23" s="72"/>
+      <c r="Y23" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="Z23" s="67"/>
+      <c r="Z23" s="72"/>
       <c r="AD23" s="11"/>
       <c r="AE23" s="5"/>
       <c r="AF23" s="3"/>
@@ -3472,6 +3488,7 @@
       <c r="AM23" s="39" t="s">
         <v>105</v>
       </c>
+      <c r="AN23" s="175"/>
       <c r="AO23" s="38" t="s">
         <v>69</v>
       </c>
@@ -3499,51 +3516,51 @@
       <c r="BH23" s="35"/>
     </row>
     <row r="24" spans="1:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="76" t="s">
+      <c r="A24" s="81" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="90"/>
-      <c r="C24" s="86"/>
-      <c r="D24" s="87"/>
-      <c r="E24" s="88"/>
-      <c r="F24" s="87"/>
-      <c r="G24" s="88"/>
-      <c r="H24" s="89"/>
-      <c r="I24" s="72" t="s">
+      <c r="B24" s="115"/>
+      <c r="C24" s="113"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="68"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="68"/>
+      <c r="H24" s="70"/>
+      <c r="I24" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="J24" s="73"/>
-      <c r="K24" s="74"/>
-      <c r="L24" s="74"/>
-      <c r="M24" s="75" t="s">
+      <c r="J24" s="67"/>
+      <c r="K24" s="65"/>
+      <c r="L24" s="65"/>
+      <c r="M24" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="N24" s="73"/>
-      <c r="O24" s="74"/>
-      <c r="P24" s="74"/>
+      <c r="N24" s="67"/>
+      <c r="O24" s="65"/>
+      <c r="P24" s="65"/>
       <c r="R24" s="23"/>
-      <c r="S24" s="76" t="s">
+      <c r="S24" s="81" t="s">
         <v>112</v>
       </c>
-      <c r="T24" s="90"/>
-      <c r="U24" s="86"/>
-      <c r="V24" s="87"/>
-      <c r="W24" s="88"/>
-      <c r="X24" s="87"/>
-      <c r="Y24" s="88"/>
-      <c r="Z24" s="89"/>
-      <c r="AA24" s="72" t="s">
+      <c r="T24" s="115"/>
+      <c r="U24" s="113"/>
+      <c r="V24" s="69"/>
+      <c r="W24" s="68"/>
+      <c r="X24" s="69"/>
+      <c r="Y24" s="68"/>
+      <c r="Z24" s="70"/>
+      <c r="AA24" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="AB24" s="73"/>
-      <c r="AC24" s="74"/>
-      <c r="AD24" s="74"/>
-      <c r="AE24" s="75" t="s">
+      <c r="AB24" s="67"/>
+      <c r="AC24" s="65"/>
+      <c r="AD24" s="65"/>
+      <c r="AE24" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="AF24" s="73"/>
-      <c r="AG24" s="74"/>
-      <c r="AH24" s="74"/>
+      <c r="AF24" s="67"/>
+      <c r="AG24" s="65"/>
+      <c r="AH24" s="65"/>
       <c r="AJ24" s="40" t="s">
         <v>52</v>
       </c>
@@ -3553,6 +3570,7 @@
       <c r="AM24" s="39" t="s">
         <v>104</v>
       </c>
+      <c r="AN24" s="175"/>
       <c r="AO24" s="38" t="s">
         <v>70</v>
       </c>
@@ -3580,18 +3598,18 @@
       <c r="BH24" s="35"/>
     </row>
     <row r="25" spans="1:60" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="67" t="s">
+      <c r="C25" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="D25" s="67"/>
-      <c r="E25" s="67" t="s">
+      <c r="D25" s="72"/>
+      <c r="E25" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="F25" s="67"/>
-      <c r="G25" s="67" t="s">
+      <c r="F25" s="72"/>
+      <c r="G25" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="H25" s="67"/>
+      <c r="H25" s="72"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
       <c r="L25" s="11"/>
@@ -3599,18 +3617,18 @@
       <c r="N25" s="3"/>
       <c r="O25" s="22"/>
       <c r="R25" s="23"/>
-      <c r="U25" s="67" t="s">
+      <c r="U25" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="V25" s="67"/>
-      <c r="W25" s="67" t="s">
+      <c r="V25" s="72"/>
+      <c r="W25" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="X25" s="67"/>
-      <c r="Y25" s="67" t="s">
+      <c r="X25" s="72"/>
+      <c r="Y25" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="Z25" s="67"/>
+      <c r="Z25" s="72"/>
       <c r="AB25" s="3"/>
       <c r="AC25" s="3"/>
       <c r="AD25" s="11"/>
@@ -3623,6 +3641,7 @@
       <c r="AL25" s="36" t="s">
         <v>47</v>
       </c>
+      <c r="AN25" s="175"/>
       <c r="AO25" s="38" t="s">
         <v>71</v>
       </c>
@@ -3650,54 +3669,55 @@
       <c r="BH25" s="35"/>
     </row>
     <row r="26" spans="1:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="76" t="s">
+      <c r="A26" s="81" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="90"/>
-      <c r="C26" s="86"/>
-      <c r="D26" s="87"/>
-      <c r="E26" s="88"/>
-      <c r="F26" s="87"/>
-      <c r="G26" s="88"/>
-      <c r="H26" s="89"/>
-      <c r="I26" s="72" t="s">
+      <c r="B26" s="115"/>
+      <c r="C26" s="113"/>
+      <c r="D26" s="69"/>
+      <c r="E26" s="68"/>
+      <c r="F26" s="69"/>
+      <c r="G26" s="68"/>
+      <c r="H26" s="70"/>
+      <c r="I26" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="J26" s="73"/>
-      <c r="K26" s="74"/>
-      <c r="L26" s="74"/>
-      <c r="M26" s="75" t="s">
+      <c r="J26" s="67"/>
+      <c r="K26" s="65"/>
+      <c r="L26" s="65"/>
+      <c r="M26" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="N26" s="73"/>
-      <c r="O26" s="74"/>
-      <c r="P26" s="74"/>
+      <c r="N26" s="67"/>
+      <c r="O26" s="65"/>
+      <c r="P26" s="65"/>
       <c r="R26" s="23"/>
-      <c r="S26" s="76" t="s">
+      <c r="S26" s="81" t="s">
         <v>113</v>
       </c>
-      <c r="T26" s="90"/>
-      <c r="U26" s="86"/>
-      <c r="V26" s="87"/>
-      <c r="W26" s="88"/>
-      <c r="X26" s="87"/>
-      <c r="Y26" s="88"/>
-      <c r="Z26" s="89"/>
-      <c r="AA26" s="72" t="s">
+      <c r="T26" s="115"/>
+      <c r="U26" s="113"/>
+      <c r="V26" s="69"/>
+      <c r="W26" s="68"/>
+      <c r="X26" s="69"/>
+      <c r="Y26" s="68"/>
+      <c r="Z26" s="70"/>
+      <c r="AA26" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="AB26" s="73"/>
-      <c r="AC26" s="74"/>
-      <c r="AD26" s="74"/>
-      <c r="AE26" s="75" t="s">
+      <c r="AB26" s="67"/>
+      <c r="AC26" s="65"/>
+      <c r="AD26" s="65"/>
+      <c r="AE26" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="AF26" s="73"/>
-      <c r="AG26" s="74"/>
-      <c r="AH26" s="74"/>
+      <c r="AF26" s="67"/>
+      <c r="AG26" s="65"/>
+      <c r="AH26" s="65"/>
       <c r="AJ26" s="40" t="s">
         <v>55</v>
       </c>
+      <c r="AN26" s="175"/>
       <c r="AO26" s="38" t="s">
         <v>64</v>
       </c>
@@ -3725,18 +3745,18 @@
       <c r="BH26" s="35"/>
     </row>
     <row r="27" spans="1:60" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="67" t="s">
+      <c r="C27" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="D27" s="67"/>
-      <c r="E27" s="67" t="s">
+      <c r="D27" s="72"/>
+      <c r="E27" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="F27" s="67"/>
-      <c r="G27" s="67" t="s">
+      <c r="F27" s="72"/>
+      <c r="G27" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="H27" s="67"/>
+      <c r="H27" s="72"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="11"/>
@@ -3744,18 +3764,18 @@
       <c r="N27" s="3"/>
       <c r="O27" s="22"/>
       <c r="R27" s="23"/>
-      <c r="U27" s="67" t="s">
+      <c r="U27" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="V27" s="67"/>
-      <c r="W27" s="67" t="s">
+      <c r="V27" s="72"/>
+      <c r="W27" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="X27" s="67"/>
-      <c r="Y27" s="67" t="s">
+      <c r="X27" s="72"/>
+      <c r="Y27" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="Z27" s="67"/>
+      <c r="Z27" s="72"/>
       <c r="AB27" s="3"/>
       <c r="AC27" s="3"/>
       <c r="AD27" s="11"/>
@@ -3765,6 +3785,7 @@
       <c r="AJ27" s="40" t="s">
         <v>54</v>
       </c>
+      <c r="AN27" s="175"/>
       <c r="AO27" s="38" t="s">
         <v>72</v>
       </c>
@@ -3792,54 +3813,55 @@
       <c r="BH27" s="35"/>
     </row>
     <row r="28" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="A28" s="76" t="s">
+      <c r="A28" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="90"/>
-      <c r="C28" s="86"/>
-      <c r="D28" s="87"/>
-      <c r="E28" s="88"/>
-      <c r="F28" s="87"/>
-      <c r="G28" s="88"/>
-      <c r="H28" s="89"/>
-      <c r="I28" s="72" t="s">
+      <c r="B28" s="115"/>
+      <c r="C28" s="113"/>
+      <c r="D28" s="69"/>
+      <c r="E28" s="68"/>
+      <c r="F28" s="69"/>
+      <c r="G28" s="68"/>
+      <c r="H28" s="70"/>
+      <c r="I28" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="J28" s="73"/>
-      <c r="K28" s="74"/>
-      <c r="L28" s="74"/>
-      <c r="M28" s="75" t="s">
+      <c r="J28" s="67"/>
+      <c r="K28" s="65"/>
+      <c r="L28" s="65"/>
+      <c r="M28" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="N28" s="73"/>
-      <c r="O28" s="74"/>
-      <c r="P28" s="74"/>
+      <c r="N28" s="67"/>
+      <c r="O28" s="65"/>
+      <c r="P28" s="65"/>
       <c r="R28" s="23"/>
-      <c r="S28" s="76" t="s">
+      <c r="S28" s="81" t="s">
         <v>114</v>
       </c>
-      <c r="T28" s="90"/>
-      <c r="U28" s="86"/>
-      <c r="V28" s="87"/>
-      <c r="W28" s="88"/>
-      <c r="X28" s="87"/>
-      <c r="Y28" s="88"/>
-      <c r="Z28" s="89"/>
-      <c r="AA28" s="72" t="s">
+      <c r="T28" s="115"/>
+      <c r="U28" s="113"/>
+      <c r="V28" s="69"/>
+      <c r="W28" s="68"/>
+      <c r="X28" s="69"/>
+      <c r="Y28" s="68"/>
+      <c r="Z28" s="70"/>
+      <c r="AA28" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="AB28" s="73"/>
-      <c r="AC28" s="74"/>
-      <c r="AD28" s="74"/>
-      <c r="AE28" s="75" t="s">
+      <c r="AB28" s="67"/>
+      <c r="AC28" s="65"/>
+      <c r="AD28" s="65"/>
+      <c r="AE28" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="AF28" s="73"/>
-      <c r="AG28" s="74"/>
-      <c r="AH28" s="74"/>
+      <c r="AF28" s="67"/>
+      <c r="AG28" s="65"/>
+      <c r="AH28" s="65"/>
       <c r="AJ28" s="40" t="s">
         <v>56</v>
       </c>
+      <c r="AN28" s="175"/>
       <c r="AO28" s="38">
         <v>10</v>
       </c>
@@ -3867,18 +3889,18 @@
       <c r="BH28" s="35"/>
     </row>
     <row r="29" spans="1:60" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C29" s="67" t="s">
+      <c r="C29" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="D29" s="67"/>
-      <c r="E29" s="67" t="s">
+      <c r="D29" s="72"/>
+      <c r="E29" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="F29" s="67"/>
-      <c r="G29" s="67" t="s">
+      <c r="F29" s="72"/>
+      <c r="G29" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="H29" s="67"/>
+      <c r="H29" s="72"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
@@ -3887,18 +3909,18 @@
       <c r="P29" s="24"/>
       <c r="Q29" s="3"/>
       <c r="R29" s="23"/>
-      <c r="U29" s="67" t="s">
+      <c r="U29" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="V29" s="67"/>
-      <c r="W29" s="67" t="s">
+      <c r="V29" s="72"/>
+      <c r="W29" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="X29" s="67"/>
-      <c r="Y29" s="67" t="s">
+      <c r="X29" s="72"/>
+      <c r="Y29" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="Z29" s="67"/>
+      <c r="Z29" s="72"/>
       <c r="AB29" s="3"/>
       <c r="AC29" s="3"/>
       <c r="AD29" s="3"/>
@@ -3909,6 +3931,7 @@
       <c r="AJ29" s="40" t="s">
         <v>174</v>
       </c>
+      <c r="AN29" s="175"/>
       <c r="AO29" s="38">
         <v>11</v>
       </c>
@@ -3936,24 +3959,24 @@
       <c r="BH29" s="35"/>
     </row>
     <row r="30" spans="1:60" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="118"/>
-      <c r="C30" s="118"/>
-      <c r="D30" s="118"/>
-      <c r="E30" s="118"/>
-      <c r="F30" s="118"/>
-      <c r="G30" s="118"/>
-      <c r="H30" s="118"/>
-      <c r="I30" s="118"/>
-      <c r="J30" s="118"/>
-      <c r="K30" s="118"/>
-      <c r="L30" s="118"/>
-      <c r="M30" s="118"/>
-      <c r="N30" s="118"/>
-      <c r="O30" s="118"/>
-      <c r="P30" s="118"/>
-      <c r="R30" s="124"/>
-      <c r="S30" s="124"/>
-      <c r="T30" s="124"/>
+      <c r="B30" s="114"/>
+      <c r="C30" s="114"/>
+      <c r="D30" s="114"/>
+      <c r="E30" s="114"/>
+      <c r="F30" s="114"/>
+      <c r="G30" s="114"/>
+      <c r="H30" s="114"/>
+      <c r="I30" s="114"/>
+      <c r="J30" s="114"/>
+      <c r="K30" s="114"/>
+      <c r="L30" s="114"/>
+      <c r="M30" s="114"/>
+      <c r="N30" s="114"/>
+      <c r="O30" s="114"/>
+      <c r="P30" s="114"/>
+      <c r="R30" s="143"/>
+      <c r="S30" s="143"/>
+      <c r="T30" s="143"/>
       <c r="U30" s="23"/>
       <c r="V30" s="23"/>
       <c r="W30" s="23"/>
@@ -3972,6 +3995,7 @@
       <c r="AJ30" s="40" t="s">
         <v>110</v>
       </c>
+      <c r="AN30" s="175"/>
       <c r="AO30" s="38">
         <v>12</v>
       </c>
@@ -4035,6 +4059,7 @@
       <c r="AJ31" s="40" t="s">
         <v>168</v>
       </c>
+      <c r="AN31" s="175"/>
       <c r="AO31" s="38" t="s">
         <v>130</v>
       </c>
@@ -4063,24 +4088,24 @@
       <c r="A32" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="125" t="s">
+      <c r="B32" s="144" t="s">
         <v>24</v>
       </c>
-      <c r="C32" s="126"/>
-      <c r="D32" s="126"/>
-      <c r="E32" s="126"/>
-      <c r="F32" s="126"/>
-      <c r="G32" s="126"/>
-      <c r="H32" s="126"/>
-      <c r="I32" s="126"/>
-      <c r="J32" s="126"/>
-      <c r="K32" s="126"/>
-      <c r="L32" s="126"/>
-      <c r="M32" s="126"/>
-      <c r="N32" s="126"/>
-      <c r="O32" s="126"/>
-      <c r="P32" s="126"/>
-      <c r="Q32" s="126"/>
+      <c r="C32" s="145"/>
+      <c r="D32" s="145"/>
+      <c r="E32" s="145"/>
+      <c r="F32" s="145"/>
+      <c r="G32" s="145"/>
+      <c r="H32" s="145"/>
+      <c r="I32" s="145"/>
+      <c r="J32" s="145"/>
+      <c r="K32" s="145"/>
+      <c r="L32" s="145"/>
+      <c r="M32" s="145"/>
+      <c r="N32" s="145"/>
+      <c r="O32" s="145"/>
+      <c r="P32" s="145"/>
+      <c r="Q32" s="145"/>
       <c r="R32" s="4"/>
       <c r="S32" s="44"/>
       <c r="T32" s="44"/>
@@ -4100,6 +4125,7 @@
       <c r="AH32" s="44"/>
       <c r="AI32" s="44"/>
       <c r="AJ32" s="39"/>
+      <c r="AN32" s="175"/>
       <c r="AO32" s="38" t="s">
         <v>131</v>
       </c>
@@ -4125,52 +4151,53 @@
       <c r="BH32" s="35"/>
     </row>
     <row r="33" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="A33" s="76" t="s">
+      <c r="A33" s="81" t="s">
         <v>119</v>
       </c>
-      <c r="B33" s="76"/>
-      <c r="C33" s="161" t="s">
+      <c r="B33" s="81"/>
+      <c r="C33" s="105" t="s">
         <v>50</v>
       </c>
-      <c r="D33" s="161"/>
-      <c r="E33" s="161"/>
-      <c r="F33" s="161"/>
-      <c r="G33" s="161"/>
-      <c r="H33" s="161"/>
-      <c r="I33" s="161"/>
+      <c r="D33" s="105"/>
+      <c r="E33" s="105"/>
+      <c r="F33" s="105"/>
+      <c r="G33" s="105"/>
+      <c r="H33" s="105"/>
+      <c r="I33" s="105"/>
       <c r="J33" s="3"/>
-      <c r="K33" s="122" t="s">
+      <c r="K33" s="140" t="s">
         <v>120</v>
       </c>
-      <c r="L33" s="123"/>
-      <c r="M33" s="123"/>
-      <c r="N33" s="123"/>
-      <c r="O33" s="123"/>
-      <c r="P33" s="123"/>
-      <c r="Q33" s="123"/>
-      <c r="R33" s="64"/>
-      <c r="S33" s="120" t="s">
+      <c r="L33" s="141"/>
+      <c r="M33" s="141"/>
+      <c r="N33" s="141"/>
+      <c r="O33" s="141"/>
+      <c r="P33" s="141"/>
+      <c r="Q33" s="141"/>
+      <c r="R33" s="142"/>
+      <c r="S33" s="74" t="s">
         <v>121</v>
       </c>
-      <c r="T33" s="120"/>
-      <c r="U33" s="120"/>
-      <c r="V33" s="120"/>
-      <c r="W33" s="120"/>
-      <c r="X33" s="120"/>
-      <c r="Y33" s="120"/>
-      <c r="Z33" s="120"/>
+      <c r="T33" s="74"/>
+      <c r="U33" s="74"/>
+      <c r="V33" s="74"/>
+      <c r="W33" s="74"/>
+      <c r="X33" s="74"/>
+      <c r="Y33" s="74"/>
+      <c r="Z33" s="74"/>
       <c r="AA33" s="4"/>
-      <c r="AB33" s="75" t="s">
+      <c r="AB33" s="66" t="s">
         <v>122</v>
       </c>
-      <c r="AC33" s="75"/>
-      <c r="AD33" s="75"/>
-      <c r="AE33" s="75"/>
-      <c r="AF33" s="75"/>
-      <c r="AG33" s="75"/>
-      <c r="AH33" s="75"/>
-      <c r="AI33" s="75"/>
+      <c r="AC33" s="66"/>
+      <c r="AD33" s="66"/>
+      <c r="AE33" s="66"/>
+      <c r="AF33" s="66"/>
+      <c r="AG33" s="66"/>
+      <c r="AH33" s="66"/>
+      <c r="AI33" s="66"/>
       <c r="AJ33" s="39"/>
+      <c r="AN33" s="175"/>
       <c r="AO33" s="38" t="s">
         <v>132</v>
       </c>
@@ -4196,42 +4223,43 @@
       <c r="BH33" s="35"/>
     </row>
     <row r="34" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="A34" s="76"/>
-      <c r="B34" s="76"/>
-      <c r="C34" s="162"/>
-      <c r="D34" s="163"/>
-      <c r="E34" s="163"/>
-      <c r="F34" s="163"/>
-      <c r="G34" s="163"/>
-      <c r="H34" s="163"/>
-      <c r="I34" s="164"/>
+      <c r="A34" s="81"/>
+      <c r="B34" s="81"/>
+      <c r="C34" s="106"/>
+      <c r="D34" s="107"/>
+      <c r="E34" s="107"/>
+      <c r="F34" s="107"/>
+      <c r="G34" s="107"/>
+      <c r="H34" s="107"/>
+      <c r="I34" s="108"/>
       <c r="J34" s="3"/>
-      <c r="K34" s="77"/>
-      <c r="L34" s="78"/>
-      <c r="M34" s="78"/>
-      <c r="N34" s="78"/>
-      <c r="O34" s="78"/>
-      <c r="P34" s="78"/>
-      <c r="Q34" s="79"/>
+      <c r="K34" s="137"/>
+      <c r="L34" s="138"/>
+      <c r="M34" s="138"/>
+      <c r="N34" s="138"/>
+      <c r="O34" s="138"/>
+      <c r="P34" s="138"/>
+      <c r="Q34" s="139"/>
       <c r="R34" s="4"/>
-      <c r="S34" s="80"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="81"/>
-      <c r="V34" s="81"/>
-      <c r="W34" s="81"/>
-      <c r="X34" s="81"/>
-      <c r="Y34" s="81"/>
-      <c r="Z34" s="82"/>
+      <c r="S34" s="171"/>
+      <c r="T34" s="172"/>
+      <c r="U34" s="172"/>
+      <c r="V34" s="172"/>
+      <c r="W34" s="172"/>
+      <c r="X34" s="172"/>
+      <c r="Y34" s="172"/>
+      <c r="Z34" s="173"/>
       <c r="AA34" s="4"/>
-      <c r="AB34" s="154"/>
-      <c r="AC34" s="155"/>
-      <c r="AD34" s="155"/>
-      <c r="AE34" s="155"/>
-      <c r="AF34" s="155"/>
-      <c r="AG34" s="155"/>
-      <c r="AH34" s="155"/>
-      <c r="AI34" s="156"/>
+      <c r="AB34" s="98"/>
+      <c r="AC34" s="99"/>
+      <c r="AD34" s="99"/>
+      <c r="AE34" s="99"/>
+      <c r="AF34" s="99"/>
+      <c r="AG34" s="99"/>
+      <c r="AH34" s="99"/>
+      <c r="AI34" s="100"/>
       <c r="AJ34" s="39"/>
+      <c r="AN34" s="175"/>
       <c r="AO34" s="38" t="s">
         <v>133</v>
       </c>
@@ -4259,48 +4287,49 @@
     <row r="35" spans="1:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
-      <c r="C35" s="152" t="s">
+      <c r="C35" s="95" t="s">
         <v>25</v>
       </c>
-      <c r="D35" s="152"/>
-      <c r="E35" s="152"/>
-      <c r="F35" s="152"/>
-      <c r="G35" s="152"/>
-      <c r="H35" s="152"/>
-      <c r="I35" s="152"/>
+      <c r="D35" s="95"/>
+      <c r="E35" s="95"/>
+      <c r="F35" s="95"/>
+      <c r="G35" s="95"/>
+      <c r="H35" s="95"/>
+      <c r="I35" s="95"/>
       <c r="J35" s="13"/>
-      <c r="K35" s="153" t="s">
+      <c r="K35" s="96" t="s">
         <v>51</v>
       </c>
-      <c r="L35" s="153"/>
-      <c r="M35" s="153"/>
-      <c r="N35" s="153"/>
-      <c r="O35" s="153"/>
-      <c r="P35" s="153"/>
-      <c r="Q35" s="153"/>
+      <c r="L35" s="96"/>
+      <c r="M35" s="96"/>
+      <c r="N35" s="96"/>
+      <c r="O35" s="96"/>
+      <c r="P35" s="96"/>
+      <c r="Q35" s="96"/>
       <c r="R35" s="4"/>
-      <c r="S35" s="85" t="s">
+      <c r="S35" s="174" t="s">
         <v>48</v>
       </c>
-      <c r="T35" s="85"/>
-      <c r="U35" s="68"/>
-      <c r="V35" s="69"/>
-      <c r="W35" s="70" t="s">
+      <c r="T35" s="174"/>
+      <c r="U35" s="109"/>
+      <c r="V35" s="110"/>
+      <c r="W35" s="169" t="s">
         <v>49</v>
       </c>
-      <c r="X35" s="71"/>
-      <c r="Y35" s="68"/>
-      <c r="Z35" s="69"/>
+      <c r="X35" s="170"/>
+      <c r="Y35" s="109"/>
+      <c r="Z35" s="110"/>
       <c r="AA35" s="4"/>
-      <c r="AB35" s="157"/>
-      <c r="AC35" s="158"/>
-      <c r="AD35" s="158"/>
-      <c r="AE35" s="158"/>
-      <c r="AF35" s="158"/>
-      <c r="AG35" s="158"/>
-      <c r="AH35" s="158"/>
-      <c r="AI35" s="159"/>
+      <c r="AB35" s="101"/>
+      <c r="AC35" s="102"/>
+      <c r="AD35" s="102"/>
+      <c r="AE35" s="102"/>
+      <c r="AF35" s="102"/>
+      <c r="AG35" s="102"/>
+      <c r="AH35" s="102"/>
+      <c r="AI35" s="103"/>
       <c r="AJ35" s="39"/>
+      <c r="AN35" s="175"/>
       <c r="AO35" s="38" t="s">
         <v>156</v>
       </c>
@@ -4335,24 +4364,24 @@
       <c r="H36" s="49"/>
       <c r="I36" s="49"/>
       <c r="J36" s="49"/>
-      <c r="K36" s="96"/>
-      <c r="L36" s="96"/>
-      <c r="M36" s="96"/>
-      <c r="N36" s="96"/>
-      <c r="O36" s="96"/>
-      <c r="P36" s="96"/>
-      <c r="Q36" s="96"/>
+      <c r="K36" s="97"/>
+      <c r="L36" s="97"/>
+      <c r="M36" s="97"/>
+      <c r="N36" s="97"/>
+      <c r="O36" s="97"/>
+      <c r="P36" s="97"/>
+      <c r="Q36" s="97"/>
       <c r="R36" s="4"/>
-      <c r="S36" s="83" t="s">
+      <c r="S36" s="150" t="s">
         <v>118</v>
       </c>
-      <c r="T36" s="84"/>
-      <c r="U36" s="84"/>
-      <c r="V36" s="84"/>
-      <c r="W36" s="84"/>
-      <c r="X36" s="84"/>
-      <c r="Y36" s="84"/>
-      <c r="Z36" s="84"/>
+      <c r="T36" s="151"/>
+      <c r="U36" s="151"/>
+      <c r="V36" s="151"/>
+      <c r="W36" s="151"/>
+      <c r="X36" s="151"/>
+      <c r="Y36" s="151"/>
+      <c r="Z36" s="151"/>
       <c r="AA36" s="4"/>
       <c r="AB36" s="44"/>
       <c r="AC36" s="44"/>
@@ -4363,6 +4392,7 @@
       <c r="AH36" s="44"/>
       <c r="AI36" s="44"/>
       <c r="AJ36" s="39"/>
+      <c r="AN36" s="175"/>
       <c r="AO36" s="38" t="s">
         <v>134</v>
       </c>
@@ -4388,48 +4418,49 @@
       <c r="BH36" s="35"/>
     </row>
     <row r="37" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="A37" s="61" t="s">
+      <c r="A37" s="164" t="s">
         <v>123</v>
       </c>
-      <c r="B37" s="62"/>
-      <c r="C37" s="63" t="s">
+      <c r="B37" s="165"/>
+      <c r="C37" s="166" t="s">
         <v>128</v>
       </c>
-      <c r="D37" s="64"/>
-      <c r="E37" s="64"/>
-      <c r="F37" s="64"/>
-      <c r="G37" s="64"/>
-      <c r="H37" s="64"/>
-      <c r="I37" s="64"/>
-      <c r="J37" s="64"/>
-      <c r="K37" s="64"/>
-      <c r="L37" s="64"/>
-      <c r="M37" s="64"/>
-      <c r="N37" s="64"/>
-      <c r="O37" s="134" t="s">
+      <c r="D37" s="142"/>
+      <c r="E37" s="142"/>
+      <c r="F37" s="142"/>
+      <c r="G37" s="142"/>
+      <c r="H37" s="142"/>
+      <c r="I37" s="142"/>
+      <c r="J37" s="142"/>
+      <c r="K37" s="142"/>
+      <c r="L37" s="142"/>
+      <c r="M37" s="142"/>
+      <c r="N37" s="142"/>
+      <c r="O37" s="92" t="s">
         <v>39</v>
       </c>
-      <c r="P37" s="135"/>
-      <c r="Q37" s="136"/>
+      <c r="P37" s="93"/>
+      <c r="Q37" s="94"/>
       <c r="R37" s="53"/>
-      <c r="S37" s="74"/>
-      <c r="T37" s="74"/>
-      <c r="U37" s="74"/>
-      <c r="V37" s="74"/>
-      <c r="W37" s="74"/>
-      <c r="X37" s="74"/>
-      <c r="Y37" s="74"/>
-      <c r="Z37" s="74"/>
+      <c r="S37" s="65"/>
+      <c r="T37" s="65"/>
+      <c r="U37" s="65"/>
+      <c r="V37" s="65"/>
+      <c r="W37" s="65"/>
+      <c r="X37" s="65"/>
+      <c r="Y37" s="65"/>
+      <c r="Z37" s="65"/>
       <c r="AA37" s="4"/>
-      <c r="AB37" s="75"/>
-      <c r="AC37" s="75"/>
-      <c r="AD37" s="75"/>
-      <c r="AE37" s="75"/>
-      <c r="AF37" s="75"/>
-      <c r="AG37" s="75"/>
-      <c r="AH37" s="75"/>
-      <c r="AI37" s="75"/>
+      <c r="AB37" s="66"/>
+      <c r="AC37" s="66"/>
+      <c r="AD37" s="66"/>
+      <c r="AE37" s="66"/>
+      <c r="AF37" s="66"/>
+      <c r="AG37" s="66"/>
+      <c r="AH37" s="66"/>
+      <c r="AI37" s="66"/>
       <c r="AJ37" s="39"/>
+      <c r="AN37" s="175"/>
       <c r="AO37" s="38" t="s">
         <v>135</v>
       </c>
@@ -4457,18 +4488,18 @@
     <row r="38" spans="1:60" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="43"/>
       <c r="B38" s="54"/>
-      <c r="C38" s="64"/>
-      <c r="D38" s="64"/>
-      <c r="E38" s="64"/>
-      <c r="F38" s="64"/>
-      <c r="G38" s="64"/>
-      <c r="H38" s="64"/>
-      <c r="I38" s="64"/>
-      <c r="J38" s="64"/>
-      <c r="K38" s="64"/>
-      <c r="L38" s="64"/>
-      <c r="M38" s="64"/>
-      <c r="N38" s="64"/>
+      <c r="C38" s="142"/>
+      <c r="D38" s="142"/>
+      <c r="E38" s="142"/>
+      <c r="F38" s="142"/>
+      <c r="G38" s="142"/>
+      <c r="H38" s="142"/>
+      <c r="I38" s="142"/>
+      <c r="J38" s="142"/>
+      <c r="K38" s="142"/>
+      <c r="L38" s="142"/>
+      <c r="M38" s="142"/>
+      <c r="N38" s="142"/>
       <c r="O38" s="46"/>
       <c r="P38" s="46"/>
       <c r="Q38" s="46"/>
@@ -4491,6 +4522,7 @@
       <c r="AH38" s="42"/>
       <c r="AI38" s="42"/>
       <c r="AJ38" s="39"/>
+      <c r="AN38" s="175"/>
       <c r="AO38" s="38" t="s">
         <v>136</v>
       </c>
@@ -4516,31 +4548,31 @@
       <c r="BH38" s="35"/>
     </row>
     <row r="39" spans="1:60" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="160"/>
-      <c r="D39" s="160"/>
-      <c r="E39" s="160"/>
-      <c r="F39" s="160"/>
-      <c r="G39" s="160"/>
-      <c r="H39" s="160"/>
-      <c r="I39" s="160"/>
+      <c r="C39" s="104"/>
+      <c r="D39" s="104"/>
+      <c r="E39" s="104"/>
+      <c r="F39" s="104"/>
+      <c r="G39" s="104"/>
+      <c r="H39" s="104"/>
+      <c r="I39" s="104"/>
       <c r="J39" s="3"/>
-      <c r="K39" s="96"/>
-      <c r="L39" s="96"/>
-      <c r="M39" s="96"/>
-      <c r="N39" s="96"/>
-      <c r="O39" s="96"/>
-      <c r="P39" s="96"/>
-      <c r="Q39" s="96"/>
-      <c r="S39" s="83" t="s">
+      <c r="K39" s="97"/>
+      <c r="L39" s="97"/>
+      <c r="M39" s="97"/>
+      <c r="N39" s="97"/>
+      <c r="O39" s="97"/>
+      <c r="P39" s="97"/>
+      <c r="Q39" s="97"/>
+      <c r="S39" s="150" t="s">
         <v>167</v>
       </c>
-      <c r="T39" s="84"/>
-      <c r="U39" s="84"/>
-      <c r="V39" s="84"/>
-      <c r="W39" s="84"/>
-      <c r="X39" s="84"/>
-      <c r="Y39" s="84"/>
-      <c r="Z39" s="84"/>
+      <c r="T39" s="151"/>
+      <c r="U39" s="151"/>
+      <c r="V39" s="151"/>
+      <c r="W39" s="151"/>
+      <c r="X39" s="151"/>
+      <c r="Y39" s="151"/>
+      <c r="Z39" s="151"/>
       <c r="AB39" s="44"/>
       <c r="AC39" s="44"/>
       <c r="AD39" s="44"/>
@@ -4550,6 +4582,7 @@
       <c r="AH39" s="44"/>
       <c r="AI39" s="44"/>
       <c r="AJ39" s="39"/>
+      <c r="AN39" s="175"/>
       <c r="AO39" s="38" t="s">
         <v>137</v>
       </c>
@@ -4575,46 +4608,47 @@
       <c r="BH39" s="35"/>
     </row>
     <row r="40" spans="1:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="61" t="s">
+      <c r="A40" s="164" t="s">
         <v>124</v>
       </c>
-      <c r="B40" s="62"/>
-      <c r="C40" s="65" t="s">
+      <c r="B40" s="165"/>
+      <c r="C40" s="167" t="s">
         <v>129</v>
       </c>
-      <c r="D40" s="66"/>
-      <c r="E40" s="66"/>
-      <c r="F40" s="66"/>
-      <c r="G40" s="66"/>
-      <c r="H40" s="66"/>
-      <c r="I40" s="66"/>
-      <c r="J40" s="66"/>
-      <c r="K40" s="66"/>
-      <c r="L40" s="66"/>
-      <c r="M40" s="66"/>
+      <c r="D40" s="168"/>
+      <c r="E40" s="168"/>
+      <c r="F40" s="168"/>
+      <c r="G40" s="168"/>
+      <c r="H40" s="168"/>
+      <c r="I40" s="168"/>
+      <c r="J40" s="168"/>
+      <c r="K40" s="168"/>
+      <c r="L40" s="168"/>
+      <c r="M40" s="168"/>
       <c r="N40" s="55"/>
-      <c r="O40" s="134" t="s">
+      <c r="O40" s="92" t="s">
         <v>39</v>
       </c>
-      <c r="P40" s="135"/>
-      <c r="Q40" s="136"/>
-      <c r="S40" s="86"/>
-      <c r="T40" s="89"/>
-      <c r="U40" s="88"/>
-      <c r="V40" s="89"/>
-      <c r="W40" s="88"/>
-      <c r="X40" s="89"/>
-      <c r="Y40" s="88"/>
-      <c r="Z40" s="89"/>
-      <c r="AB40" s="67"/>
-      <c r="AC40" s="67"/>
-      <c r="AD40" s="67"/>
-      <c r="AE40" s="67"/>
-      <c r="AF40" s="67"/>
-      <c r="AG40" s="67"/>
-      <c r="AH40" s="67"/>
-      <c r="AI40" s="67"/>
+      <c r="P40" s="93"/>
+      <c r="Q40" s="94"/>
+      <c r="S40" s="113"/>
+      <c r="T40" s="70"/>
+      <c r="U40" s="68"/>
+      <c r="V40" s="70"/>
+      <c r="W40" s="68"/>
+      <c r="X40" s="70"/>
+      <c r="Y40" s="68"/>
+      <c r="Z40" s="70"/>
+      <c r="AB40" s="72"/>
+      <c r="AC40" s="72"/>
+      <c r="AD40" s="72"/>
+      <c r="AE40" s="72"/>
+      <c r="AF40" s="72"/>
+      <c r="AG40" s="72"/>
+      <c r="AH40" s="72"/>
+      <c r="AI40" s="72"/>
       <c r="AJ40" s="39"/>
+      <c r="AN40" s="175"/>
       <c r="AO40" s="38" t="s">
         <v>157</v>
       </c>
@@ -4676,6 +4710,7 @@
       <c r="AH41" s="15"/>
       <c r="AI41" s="15"/>
       <c r="AJ41" s="39"/>
+      <c r="AN41" s="175"/>
       <c r="AO41" s="38" t="s">
         <v>158</v>
       </c>
@@ -4704,24 +4739,25 @@
       <c r="A42" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B42" s="118" t="s">
+      <c r="B42" s="114" t="s">
         <v>26</v>
       </c>
-      <c r="C42" s="118"/>
-      <c r="D42" s="118"/>
-      <c r="E42" s="118"/>
-      <c r="F42" s="118"/>
-      <c r="G42" s="118"/>
-      <c r="H42" s="118"/>
-      <c r="I42" s="118"/>
-      <c r="J42" s="118"/>
-      <c r="K42" s="118"/>
-      <c r="L42" s="118"/>
-      <c r="M42" s="118"/>
-      <c r="N42" s="118"/>
-      <c r="O42" s="118"/>
-      <c r="P42" s="118"/>
+      <c r="C42" s="114"/>
+      <c r="D42" s="114"/>
+      <c r="E42" s="114"/>
+      <c r="F42" s="114"/>
+      <c r="G42" s="114"/>
+      <c r="H42" s="114"/>
+      <c r="I42" s="114"/>
+      <c r="J42" s="114"/>
+      <c r="K42" s="114"/>
+      <c r="L42" s="114"/>
+      <c r="M42" s="114"/>
+      <c r="N42" s="114"/>
+      <c r="O42" s="114"/>
+      <c r="P42" s="114"/>
       <c r="AJ42" s="39"/>
+      <c r="AN42" s="175"/>
       <c r="AO42" s="38" t="s">
         <v>159</v>
       </c>
@@ -4747,39 +4783,40 @@
       <c r="BH42" s="35"/>
     </row>
     <row r="43" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="B43" s="103"/>
-      <c r="C43" s="104"/>
-      <c r="D43" s="104"/>
-      <c r="E43" s="104"/>
-      <c r="F43" s="104"/>
-      <c r="G43" s="104"/>
-      <c r="H43" s="104"/>
-      <c r="I43" s="104"/>
-      <c r="J43" s="104"/>
-      <c r="K43" s="104"/>
-      <c r="L43" s="104"/>
-      <c r="M43" s="104"/>
-      <c r="N43" s="104"/>
-      <c r="O43" s="105"/>
-      <c r="Q43" s="109"/>
-      <c r="R43" s="110"/>
-      <c r="S43" s="110"/>
-      <c r="T43" s="110"/>
-      <c r="U43" s="110"/>
-      <c r="V43" s="110"/>
-      <c r="W43" s="110"/>
-      <c r="X43" s="111"/>
-      <c r="Z43" s="103"/>
-      <c r="AA43" s="104"/>
-      <c r="AB43" s="104"/>
-      <c r="AC43" s="104"/>
-      <c r="AD43" s="104"/>
-      <c r="AE43" s="104"/>
-      <c r="AF43" s="104"/>
-      <c r="AG43" s="104"/>
-      <c r="AH43" s="104"/>
-      <c r="AI43" s="105"/>
+      <c r="B43" s="86"/>
+      <c r="C43" s="87"/>
+      <c r="D43" s="87"/>
+      <c r="E43" s="87"/>
+      <c r="F43" s="87"/>
+      <c r="G43" s="87"/>
+      <c r="H43" s="87"/>
+      <c r="I43" s="87"/>
+      <c r="J43" s="87"/>
+      <c r="K43" s="87"/>
+      <c r="L43" s="87"/>
+      <c r="M43" s="87"/>
+      <c r="N43" s="87"/>
+      <c r="O43" s="88"/>
+      <c r="Q43" s="154"/>
+      <c r="R43" s="155"/>
+      <c r="S43" s="155"/>
+      <c r="T43" s="155"/>
+      <c r="U43" s="155"/>
+      <c r="V43" s="155"/>
+      <c r="W43" s="155"/>
+      <c r="X43" s="156"/>
+      <c r="Z43" s="86"/>
+      <c r="AA43" s="87"/>
+      <c r="AB43" s="87"/>
+      <c r="AC43" s="87"/>
+      <c r="AD43" s="87"/>
+      <c r="AE43" s="87"/>
+      <c r="AF43" s="87"/>
+      <c r="AG43" s="87"/>
+      <c r="AH43" s="87"/>
+      <c r="AI43" s="88"/>
       <c r="AJ43" s="39"/>
+      <c r="AN43" s="175"/>
       <c r="AO43" s="38" t="s">
         <v>160</v>
       </c>
@@ -4803,39 +4840,40 @@
       <c r="BH43" s="35"/>
     </row>
     <row r="44" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="B44" s="106"/>
-      <c r="C44" s="107"/>
-      <c r="D44" s="107"/>
-      <c r="E44" s="107"/>
-      <c r="F44" s="107"/>
-      <c r="G44" s="107"/>
-      <c r="H44" s="107"/>
-      <c r="I44" s="107"/>
-      <c r="J44" s="107"/>
-      <c r="K44" s="107"/>
-      <c r="L44" s="107"/>
-      <c r="M44" s="107"/>
-      <c r="N44" s="107"/>
-      <c r="O44" s="108"/>
-      <c r="Q44" s="112"/>
-      <c r="R44" s="113"/>
-      <c r="S44" s="113"/>
-      <c r="T44" s="113"/>
-      <c r="U44" s="113"/>
-      <c r="V44" s="113"/>
-      <c r="W44" s="113"/>
-      <c r="X44" s="114"/>
-      <c r="Z44" s="106"/>
-      <c r="AA44" s="107"/>
-      <c r="AB44" s="107"/>
-      <c r="AC44" s="107"/>
-      <c r="AD44" s="107"/>
-      <c r="AE44" s="107"/>
-      <c r="AF44" s="107"/>
-      <c r="AG44" s="107"/>
-      <c r="AH44" s="107"/>
-      <c r="AI44" s="108"/>
+      <c r="B44" s="89"/>
+      <c r="C44" s="90"/>
+      <c r="D44" s="90"/>
+      <c r="E44" s="90"/>
+      <c r="F44" s="90"/>
+      <c r="G44" s="90"/>
+      <c r="H44" s="90"/>
+      <c r="I44" s="90"/>
+      <c r="J44" s="90"/>
+      <c r="K44" s="90"/>
+      <c r="L44" s="90"/>
+      <c r="M44" s="90"/>
+      <c r="N44" s="90"/>
+      <c r="O44" s="91"/>
+      <c r="Q44" s="157"/>
+      <c r="R44" s="158"/>
+      <c r="S44" s="158"/>
+      <c r="T44" s="158"/>
+      <c r="U44" s="158"/>
+      <c r="V44" s="158"/>
+      <c r="W44" s="158"/>
+      <c r="X44" s="159"/>
+      <c r="Z44" s="89"/>
+      <c r="AA44" s="90"/>
+      <c r="AB44" s="90"/>
+      <c r="AC44" s="90"/>
+      <c r="AD44" s="90"/>
+      <c r="AE44" s="90"/>
+      <c r="AF44" s="90"/>
+      <c r="AG44" s="90"/>
+      <c r="AH44" s="90"/>
+      <c r="AI44" s="91"/>
       <c r="AJ44" s="39"/>
+      <c r="AN44" s="175"/>
       <c r="AO44" s="38" t="s">
         <v>161</v>
       </c>
@@ -4846,43 +4884,44 @@
       <c r="AS44" s="38"/>
     </row>
     <row r="45" spans="1:60" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="95" t="s">
+      <c r="B45" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="C45" s="95"/>
-      <c r="D45" s="95"/>
-      <c r="E45" s="95"/>
-      <c r="F45" s="95"/>
-      <c r="G45" s="95"/>
-      <c r="H45" s="95"/>
-      <c r="I45" s="95"/>
-      <c r="J45" s="95"/>
-      <c r="K45" s="95"/>
-      <c r="L45" s="95"/>
-      <c r="M45" s="95"/>
-      <c r="N45" s="95"/>
-      <c r="O45" s="95"/>
-      <c r="Q45" s="115"/>
-      <c r="R45" s="116"/>
-      <c r="S45" s="116"/>
-      <c r="T45" s="116"/>
-      <c r="U45" s="116"/>
-      <c r="V45" s="116"/>
-      <c r="W45" s="116"/>
-      <c r="X45" s="117"/>
-      <c r="Z45" s="67" t="s">
+      <c r="C45" s="136"/>
+      <c r="D45" s="136"/>
+      <c r="E45" s="136"/>
+      <c r="F45" s="136"/>
+      <c r="G45" s="136"/>
+      <c r="H45" s="136"/>
+      <c r="I45" s="136"/>
+      <c r="J45" s="136"/>
+      <c r="K45" s="136"/>
+      <c r="L45" s="136"/>
+      <c r="M45" s="136"/>
+      <c r="N45" s="136"/>
+      <c r="O45" s="136"/>
+      <c r="Q45" s="160"/>
+      <c r="R45" s="161"/>
+      <c r="S45" s="161"/>
+      <c r="T45" s="161"/>
+      <c r="U45" s="161"/>
+      <c r="V45" s="161"/>
+      <c r="W45" s="161"/>
+      <c r="X45" s="162"/>
+      <c r="Z45" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="AA45" s="67"/>
-      <c r="AB45" s="67"/>
-      <c r="AC45" s="67"/>
-      <c r="AD45" s="67"/>
-      <c r="AE45" s="67"/>
-      <c r="AF45" s="67"/>
-      <c r="AG45" s="67"/>
-      <c r="AH45" s="67"/>
-      <c r="AI45" s="67"/>
+      <c r="AA45" s="72"/>
+      <c r="AB45" s="72"/>
+      <c r="AC45" s="72"/>
+      <c r="AD45" s="72"/>
+      <c r="AE45" s="72"/>
+      <c r="AF45" s="72"/>
+      <c r="AG45" s="72"/>
+      <c r="AH45" s="72"/>
+      <c r="AI45" s="72"/>
       <c r="AJ45" s="39"/>
+      <c r="AN45" s="175"/>
       <c r="AO45" s="38" t="s">
         <v>162</v>
       </c>
@@ -4897,17 +4936,18 @@
       <c r="O46" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="Q46" s="119" t="s">
+      <c r="Q46" s="163" t="s">
         <v>29</v>
       </c>
-      <c r="R46" s="119"/>
-      <c r="S46" s="119"/>
-      <c r="T46" s="119"/>
-      <c r="U46" s="119"/>
-      <c r="V46" s="119"/>
-      <c r="W46" s="119"/>
-      <c r="X46" s="119"/>
+      <c r="R46" s="163"/>
+      <c r="S46" s="163"/>
+      <c r="T46" s="163"/>
+      <c r="U46" s="163"/>
+      <c r="V46" s="163"/>
+      <c r="W46" s="163"/>
+      <c r="X46" s="163"/>
       <c r="AJ46" s="39"/>
+      <c r="AN46" s="175"/>
       <c r="AO46" s="38" t="s">
         <v>163</v>
       </c>
@@ -4940,28 +4980,29 @@
       <c r="P47" s="28"/>
       <c r="Q47" s="28"/>
       <c r="R47" s="28"/>
-      <c r="S47" s="98"/>
-      <c r="T47" s="99"/>
-      <c r="U47" s="99"/>
-      <c r="V47" s="100"/>
+      <c r="S47" s="85"/>
+      <c r="T47" s="152"/>
+      <c r="U47" s="152"/>
+      <c r="V47" s="153"/>
       <c r="W47" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="X47" s="101"/>
-      <c r="Y47" s="98"/>
-      <c r="Z47" s="169"/>
-      <c r="AA47" s="170"/>
-      <c r="AB47" s="100"/>
-      <c r="AC47" s="101"/>
+      <c r="X47" s="84"/>
+      <c r="Y47" s="85"/>
+      <c r="Z47" s="82"/>
+      <c r="AA47" s="83"/>
+      <c r="AB47" s="153"/>
+      <c r="AC47" s="84"/>
       <c r="AD47" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="AE47" s="166"/>
-      <c r="AF47" s="167"/>
-      <c r="AG47" s="167"/>
-      <c r="AH47" s="167"/>
-      <c r="AI47" s="168"/>
+      <c r="AE47" s="76"/>
+      <c r="AF47" s="77"/>
+      <c r="AG47" s="77"/>
+      <c r="AH47" s="77"/>
+      <c r="AI47" s="78"/>
       <c r="AJ47" s="39"/>
+      <c r="AN47" s="175"/>
       <c r="AO47" s="38" t="s">
         <v>164</v>
       </c>
@@ -4973,32 +5014,33 @@
       <c r="AS47" s="38"/>
     </row>
     <row r="48" spans="1:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="S48" s="97" t="s">
+      <c r="S48" s="79" t="s">
         <v>12</v>
       </c>
-      <c r="T48" s="97"/>
-      <c r="U48" s="97"/>
-      <c r="V48" s="97"/>
-      <c r="X48" s="97" t="s">
+      <c r="T48" s="79"/>
+      <c r="U48" s="79"/>
+      <c r="V48" s="79"/>
+      <c r="X48" s="79" t="s">
         <v>17</v>
       </c>
-      <c r="Y48" s="97"/>
-      <c r="Z48" s="97" t="s">
+      <c r="Y48" s="79"/>
+      <c r="Z48" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="AA48" s="97"/>
-      <c r="AB48" s="97" t="s">
+      <c r="AA48" s="79"/>
+      <c r="AB48" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="AC48" s="97"/>
-      <c r="AE48" s="102" t="s">
+      <c r="AC48" s="79"/>
+      <c r="AE48" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="AF48" s="102"/>
-      <c r="AG48" s="102"/>
-      <c r="AH48" s="102"/>
-      <c r="AI48" s="102"/>
+      <c r="AF48" s="80"/>
+      <c r="AG48" s="80"/>
+      <c r="AH48" s="80"/>
+      <c r="AI48" s="80"/>
       <c r="AJ48" s="39"/>
+      <c r="AN48" s="175"/>
       <c r="AO48" s="38" t="s">
         <v>165</v>
       </c>
@@ -5027,22 +5069,23 @@
       <c r="P49" s="6"/>
       <c r="Q49" s="6"/>
       <c r="R49" s="6"/>
-      <c r="S49" s="102"/>
-      <c r="T49" s="102"/>
-      <c r="U49" s="102"/>
-      <c r="V49" s="102"/>
+      <c r="S49" s="80"/>
+      <c r="T49" s="80"/>
+      <c r="U49" s="80"/>
+      <c r="V49" s="80"/>
       <c r="Y49" s="3"/>
       <c r="Z49" s="3"/>
       <c r="AA49" s="3"/>
       <c r="AB49" s="3"/>
       <c r="AC49" s="3"/>
       <c r="AD49" s="27"/>
-      <c r="AE49" s="102"/>
-      <c r="AF49" s="102"/>
-      <c r="AG49" s="102"/>
-      <c r="AH49" s="102"/>
-      <c r="AI49" s="102"/>
+      <c r="AE49" s="80"/>
+      <c r="AF49" s="80"/>
+      <c r="AG49" s="80"/>
+      <c r="AH49" s="80"/>
+      <c r="AI49" s="80"/>
       <c r="AJ49" s="39"/>
+      <c r="AN49" s="175"/>
       <c r="AO49" s="38" t="s">
         <v>166</v>
       </c>
@@ -5057,19 +5100,19 @@
       <c r="A50" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B50" s="118" t="s">
+      <c r="B50" s="114" t="s">
         <v>31</v>
       </c>
-      <c r="C50" s="118"/>
-      <c r="D50" s="118"/>
-      <c r="E50" s="118"/>
-      <c r="F50" s="118"/>
-      <c r="G50" s="118"/>
-      <c r="H50" s="118"/>
-      <c r="I50" s="118"/>
-      <c r="J50" s="118"/>
-      <c r="K50" s="118"/>
-      <c r="L50" s="118"/>
+      <c r="C50" s="114"/>
+      <c r="D50" s="114"/>
+      <c r="E50" s="114"/>
+      <c r="F50" s="114"/>
+      <c r="G50" s="114"/>
+      <c r="H50" s="114"/>
+      <c r="I50" s="114"/>
+      <c r="J50" s="114"/>
+      <c r="K50" s="114"/>
+      <c r="L50" s="114"/>
       <c r="Z50" s="3"/>
       <c r="AA50" s="3"/>
       <c r="AB50" s="3"/>
@@ -5080,6 +5123,7 @@
       <c r="AH50" s="3"/>
       <c r="AI50" s="3"/>
       <c r="AJ50" s="39"/>
+      <c r="AN50" s="175"/>
       <c r="AO50" s="38"/>
       <c r="AP50" s="38"/>
       <c r="AQ50" s="38" t="s">
@@ -5090,6 +5134,7 @@
     </row>
     <row r="51" spans="1:45" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AJ51" s="39"/>
+      <c r="AN51" s="175"/>
       <c r="AO51" s="38"/>
       <c r="AP51" s="38"/>
       <c r="AQ51" s="38" t="s">
@@ -5099,10 +5144,10 @@
       <c r="AS51" s="38"/>
     </row>
     <row r="52" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A52" s="76" t="s">
+      <c r="A52" s="81" t="s">
         <v>32</v>
       </c>
-      <c r="B52" s="76"/>
+      <c r="B52" s="81"/>
       <c r="C52" s="12" t="s">
         <v>33</v>
       </c>
@@ -5133,21 +5178,22 @@
       </c>
       <c r="S52" s="31"/>
       <c r="T52" s="33"/>
-      <c r="X52" s="76" t="s">
+      <c r="X52" s="81" t="s">
         <v>127</v>
       </c>
-      <c r="Y52" s="90"/>
-      <c r="Z52" s="103"/>
-      <c r="AA52" s="104"/>
-      <c r="AB52" s="104"/>
-      <c r="AC52" s="104"/>
-      <c r="AD52" s="104"/>
-      <c r="AE52" s="104"/>
-      <c r="AF52" s="104"/>
-      <c r="AG52" s="104"/>
-      <c r="AH52" s="104"/>
-      <c r="AI52" s="105"/>
+      <c r="Y52" s="115"/>
+      <c r="Z52" s="86"/>
+      <c r="AA52" s="87"/>
+      <c r="AB52" s="87"/>
+      <c r="AC52" s="87"/>
+      <c r="AD52" s="87"/>
+      <c r="AE52" s="87"/>
+      <c r="AF52" s="87"/>
+      <c r="AG52" s="87"/>
+      <c r="AH52" s="87"/>
+      <c r="AI52" s="88"/>
       <c r="AJ52" s="39"/>
+      <c r="AN52" s="175"/>
       <c r="AO52" s="38"/>
       <c r="AP52" s="38"/>
       <c r="AQ52" s="38" t="s">
@@ -5158,33 +5204,34 @@
     </row>
     <row r="53" spans="1:45" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G53" s="3"/>
-      <c r="H53" s="165" t="s">
+      <c r="H53" s="75" t="s">
         <v>37</v>
       </c>
-      <c r="I53" s="165"/>
-      <c r="J53" s="165"/>
-      <c r="L53" s="67" t="s">
+      <c r="I53" s="75"/>
+      <c r="J53" s="75"/>
+      <c r="L53" s="72" t="s">
         <v>38</v>
       </c>
-      <c r="M53" s="67"/>
-      <c r="N53" s="67"/>
-      <c r="O53" s="67"/>
-      <c r="P53" s="67"/>
-      <c r="Q53" s="67"/>
-      <c r="R53" s="67"/>
-      <c r="S53" s="67"/>
-      <c r="T53" s="67"/>
-      <c r="Z53" s="106"/>
-      <c r="AA53" s="107"/>
-      <c r="AB53" s="107"/>
-      <c r="AC53" s="107"/>
-      <c r="AD53" s="107"/>
-      <c r="AE53" s="107"/>
-      <c r="AF53" s="107"/>
-      <c r="AG53" s="107"/>
-      <c r="AH53" s="107"/>
-      <c r="AI53" s="108"/>
+      <c r="M53" s="72"/>
+      <c r="N53" s="72"/>
+      <c r="O53" s="72"/>
+      <c r="P53" s="72"/>
+      <c r="Q53" s="72"/>
+      <c r="R53" s="72"/>
+      <c r="S53" s="72"/>
+      <c r="T53" s="72"/>
+      <c r="Z53" s="89"/>
+      <c r="AA53" s="90"/>
+      <c r="AB53" s="90"/>
+      <c r="AC53" s="90"/>
+      <c r="AD53" s="90"/>
+      <c r="AE53" s="90"/>
+      <c r="AF53" s="90"/>
+      <c r="AG53" s="90"/>
+      <c r="AH53" s="90"/>
+      <c r="AI53" s="91"/>
       <c r="AJ53" s="39"/>
+      <c r="AN53" s="175"/>
       <c r="AO53" s="38"/>
       <c r="AP53" s="38"/>
       <c r="AQ53" s="38" t="s">
@@ -5194,11 +5241,11 @@
       <c r="AS53" s="38"/>
     </row>
     <row r="54" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="C54" s="118" t="s">
+      <c r="C54" s="114" t="s">
         <v>33</v>
       </c>
-      <c r="D54" s="118"/>
-      <c r="E54" s="118"/>
+      <c r="D54" s="114"/>
+      <c r="E54" s="114"/>
       <c r="F54" s="7">
         <v>8</v>
       </c>
@@ -5224,19 +5271,20 @@
       </c>
       <c r="S54" s="31"/>
       <c r="T54" s="33"/>
-      <c r="Z54" s="67" t="s">
+      <c r="Z54" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="AA54" s="67"/>
-      <c r="AB54" s="67"/>
-      <c r="AC54" s="67"/>
-      <c r="AD54" s="67"/>
-      <c r="AE54" s="67"/>
-      <c r="AF54" s="67"/>
-      <c r="AG54" s="67"/>
-      <c r="AH54" s="67"/>
-      <c r="AI54" s="67"/>
+      <c r="AA54" s="72"/>
+      <c r="AB54" s="72"/>
+      <c r="AC54" s="72"/>
+      <c r="AD54" s="72"/>
+      <c r="AE54" s="72"/>
+      <c r="AF54" s="72"/>
+      <c r="AG54" s="72"/>
+      <c r="AH54" s="72"/>
+      <c r="AI54" s="72"/>
       <c r="AJ54" s="39"/>
+      <c r="AN54" s="175"/>
       <c r="AO54" s="38"/>
       <c r="AP54" s="38"/>
       <c r="AQ54" s="38" t="s">
@@ -5247,67 +5295,70 @@
     </row>
     <row r="55" spans="1:45" x14ac:dyDescent="0.25">
       <c r="G55" s="3"/>
-      <c r="H55" s="95" t="s">
+      <c r="H55" s="136" t="s">
         <v>37</v>
       </c>
-      <c r="I55" s="95"/>
-      <c r="J55" s="95"/>
-      <c r="L55" s="67" t="s">
+      <c r="I55" s="136"/>
+      <c r="J55" s="136"/>
+      <c r="L55" s="72" t="s">
         <v>38</v>
       </c>
-      <c r="M55" s="67"/>
-      <c r="N55" s="67"/>
-      <c r="O55" s="67"/>
-      <c r="P55" s="67"/>
-      <c r="Q55" s="67"/>
-      <c r="R55" s="67"/>
-      <c r="S55" s="67"/>
-      <c r="T55" s="67"/>
+      <c r="M55" s="72"/>
+      <c r="N55" s="72"/>
+      <c r="O55" s="72"/>
+      <c r="P55" s="72"/>
+      <c r="Q55" s="72"/>
+      <c r="R55" s="72"/>
+      <c r="S55" s="72"/>
+      <c r="T55" s="72"/>
       <c r="AJ55" s="39"/>
+      <c r="AN55" s="175"/>
       <c r="AO55" s="38"/>
       <c r="AP55" s="38"/>
-      <c r="AQ55" s="38"/>
+      <c r="AQ55" s="38" t="s">
+        <v>179</v>
+      </c>
       <c r="AR55" s="38"/>
       <c r="AS55" s="38"/>
     </row>
     <row r="56" spans="1:45" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="93" t="s">
+      <c r="A56" s="148" t="s">
         <v>57</v>
       </c>
-      <c r="B56" s="93"/>
-      <c r="C56" s="93"/>
-      <c r="D56" s="93"/>
-      <c r="E56" s="93"/>
-      <c r="F56" s="93"/>
-      <c r="G56" s="93"/>
-      <c r="H56" s="93"/>
-      <c r="I56" s="93"/>
-      <c r="J56" s="93"/>
-      <c r="K56" s="93"/>
-      <c r="L56" s="93"/>
-      <c r="M56" s="93"/>
-      <c r="N56" s="93"/>
-      <c r="O56" s="93"/>
-      <c r="P56" s="93"/>
-      <c r="Q56" s="93"/>
-      <c r="R56" s="93"/>
-      <c r="S56" s="93"/>
-      <c r="T56" s="93"/>
-      <c r="U56" s="93"/>
-      <c r="V56" s="93"/>
-      <c r="W56" s="93"/>
-      <c r="X56" s="93"/>
-      <c r="Y56" s="93"/>
-      <c r="Z56" s="93"/>
-      <c r="AA56" s="93"/>
-      <c r="AB56" s="93"/>
-      <c r="AC56" s="93"/>
-      <c r="AD56" s="93"/>
-      <c r="AE56" s="93"/>
-      <c r="AF56" s="93"/>
-      <c r="AG56" s="93"/>
-      <c r="AH56" s="93"/>
-      <c r="AI56" s="93"/>
+      <c r="B56" s="148"/>
+      <c r="C56" s="148"/>
+      <c r="D56" s="148"/>
+      <c r="E56" s="148"/>
+      <c r="F56" s="148"/>
+      <c r="G56" s="148"/>
+      <c r="H56" s="148"/>
+      <c r="I56" s="148"/>
+      <c r="J56" s="148"/>
+      <c r="K56" s="148"/>
+      <c r="L56" s="148"/>
+      <c r="M56" s="148"/>
+      <c r="N56" s="148"/>
+      <c r="O56" s="148"/>
+      <c r="P56" s="148"/>
+      <c r="Q56" s="148"/>
+      <c r="R56" s="148"/>
+      <c r="S56" s="148"/>
+      <c r="T56" s="148"/>
+      <c r="U56" s="148"/>
+      <c r="V56" s="148"/>
+      <c r="W56" s="148"/>
+      <c r="X56" s="148"/>
+      <c r="Y56" s="148"/>
+      <c r="Z56" s="148"/>
+      <c r="AA56" s="148"/>
+      <c r="AB56" s="148"/>
+      <c r="AC56" s="148"/>
+      <c r="AD56" s="148"/>
+      <c r="AE56" s="148"/>
+      <c r="AF56" s="148"/>
+      <c r="AG56" s="148"/>
+      <c r="AH56" s="148"/>
+      <c r="AI56" s="148"/>
       <c r="AJ56" s="39"/>
       <c r="AO56" s="38"/>
       <c r="AP56" s="38"/>
@@ -5316,41 +5367,41 @@
       <c r="AS56" s="38"/>
     </row>
     <row r="57" spans="1:45" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="94"/>
-      <c r="B57" s="94"/>
-      <c r="C57" s="94"/>
-      <c r="D57" s="94"/>
-      <c r="E57" s="94"/>
-      <c r="F57" s="94"/>
-      <c r="G57" s="94"/>
-      <c r="H57" s="94"/>
-      <c r="I57" s="94"/>
-      <c r="J57" s="94"/>
-      <c r="K57" s="94"/>
-      <c r="L57" s="94"/>
-      <c r="M57" s="94"/>
-      <c r="N57" s="94"/>
-      <c r="O57" s="94"/>
-      <c r="P57" s="94"/>
-      <c r="Q57" s="94"/>
-      <c r="R57" s="94"/>
-      <c r="S57" s="94"/>
-      <c r="T57" s="94"/>
-      <c r="U57" s="94"/>
-      <c r="V57" s="94"/>
-      <c r="W57" s="94"/>
-      <c r="X57" s="94"/>
-      <c r="Y57" s="94"/>
-      <c r="Z57" s="94"/>
-      <c r="AA57" s="94"/>
-      <c r="AB57" s="94"/>
-      <c r="AC57" s="94"/>
-      <c r="AD57" s="94"/>
-      <c r="AE57" s="94"/>
-      <c r="AF57" s="94"/>
-      <c r="AG57" s="94"/>
-      <c r="AH57" s="94"/>
-      <c r="AI57" s="94"/>
+      <c r="A57" s="149"/>
+      <c r="B57" s="149"/>
+      <c r="C57" s="149"/>
+      <c r="D57" s="149"/>
+      <c r="E57" s="149"/>
+      <c r="F57" s="149"/>
+      <c r="G57" s="149"/>
+      <c r="H57" s="149"/>
+      <c r="I57" s="149"/>
+      <c r="J57" s="149"/>
+      <c r="K57" s="149"/>
+      <c r="L57" s="149"/>
+      <c r="M57" s="149"/>
+      <c r="N57" s="149"/>
+      <c r="O57" s="149"/>
+      <c r="P57" s="149"/>
+      <c r="Q57" s="149"/>
+      <c r="R57" s="149"/>
+      <c r="S57" s="149"/>
+      <c r="T57" s="149"/>
+      <c r="U57" s="149"/>
+      <c r="V57" s="149"/>
+      <c r="W57" s="149"/>
+      <c r="X57" s="149"/>
+      <c r="Y57" s="149"/>
+      <c r="Z57" s="149"/>
+      <c r="AA57" s="149"/>
+      <c r="AB57" s="149"/>
+      <c r="AC57" s="149"/>
+      <c r="AD57" s="149"/>
+      <c r="AE57" s="149"/>
+      <c r="AF57" s="149"/>
+      <c r="AG57" s="149"/>
+      <c r="AH57" s="149"/>
+      <c r="AI57" s="149"/>
       <c r="AJ57" s="39"/>
       <c r="AO57" s="38"/>
       <c r="AP57" s="38"/>
@@ -5359,43 +5410,43 @@
       <c r="AS57" s="38"/>
     </row>
     <row r="58" spans="1:45" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="91" t="s">
+      <c r="A58" s="146" t="s">
         <v>100</v>
       </c>
-      <c r="B58" s="91"/>
-      <c r="C58" s="91"/>
-      <c r="D58" s="91"/>
-      <c r="E58" s="91"/>
-      <c r="F58" s="91"/>
-      <c r="G58" s="91"/>
-      <c r="H58" s="91"/>
-      <c r="I58" s="91"/>
-      <c r="J58" s="91"/>
-      <c r="K58" s="91"/>
-      <c r="L58" s="91"/>
-      <c r="M58" s="91"/>
-      <c r="N58" s="91"/>
-      <c r="O58" s="91"/>
-      <c r="P58" s="91"/>
-      <c r="Q58" s="91"/>
-      <c r="R58" s="91"/>
-      <c r="S58" s="91"/>
-      <c r="T58" s="91"/>
-      <c r="U58" s="91"/>
-      <c r="V58" s="91"/>
-      <c r="W58" s="91"/>
-      <c r="X58" s="91"/>
-      <c r="Y58" s="91"/>
-      <c r="Z58" s="91"/>
-      <c r="AA58" s="91"/>
-      <c r="AB58" s="91"/>
-      <c r="AC58" s="91"/>
-      <c r="AD58" s="91"/>
-      <c r="AE58" s="91"/>
-      <c r="AF58" s="91"/>
-      <c r="AG58" s="91"/>
-      <c r="AH58" s="91"/>
-      <c r="AI58" s="91"/>
+      <c r="B58" s="146"/>
+      <c r="C58" s="146"/>
+      <c r="D58" s="146"/>
+      <c r="E58" s="146"/>
+      <c r="F58" s="146"/>
+      <c r="G58" s="146"/>
+      <c r="H58" s="146"/>
+      <c r="I58" s="146"/>
+      <c r="J58" s="146"/>
+      <c r="K58" s="146"/>
+      <c r="L58" s="146"/>
+      <c r="M58" s="146"/>
+      <c r="N58" s="146"/>
+      <c r="O58" s="146"/>
+      <c r="P58" s="146"/>
+      <c r="Q58" s="146"/>
+      <c r="R58" s="146"/>
+      <c r="S58" s="146"/>
+      <c r="T58" s="146"/>
+      <c r="U58" s="146"/>
+      <c r="V58" s="146"/>
+      <c r="W58" s="146"/>
+      <c r="X58" s="146"/>
+      <c r="Y58" s="146"/>
+      <c r="Z58" s="146"/>
+      <c r="AA58" s="146"/>
+      <c r="AB58" s="146"/>
+      <c r="AC58" s="146"/>
+      <c r="AD58" s="146"/>
+      <c r="AE58" s="146"/>
+      <c r="AF58" s="146"/>
+      <c r="AG58" s="146"/>
+      <c r="AH58" s="146"/>
+      <c r="AI58" s="146"/>
       <c r="AJ58" s="39"/>
       <c r="AO58" s="38"/>
       <c r="AP58" s="38"/>
@@ -5404,41 +5455,41 @@
       <c r="AS58" s="38"/>
     </row>
     <row r="59" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A59" s="92"/>
-      <c r="B59" s="92"/>
-      <c r="C59" s="92"/>
-      <c r="D59" s="92"/>
-      <c r="E59" s="92"/>
-      <c r="F59" s="92"/>
-      <c r="G59" s="92"/>
-      <c r="H59" s="92"/>
-      <c r="I59" s="92"/>
-      <c r="J59" s="92"/>
-      <c r="K59" s="92"/>
-      <c r="L59" s="92"/>
-      <c r="M59" s="92"/>
-      <c r="N59" s="92"/>
-      <c r="O59" s="92"/>
-      <c r="P59" s="92"/>
-      <c r="Q59" s="92"/>
-      <c r="R59" s="92"/>
-      <c r="S59" s="92"/>
-      <c r="T59" s="92"/>
-      <c r="U59" s="92"/>
-      <c r="V59" s="92"/>
-      <c r="W59" s="92"/>
-      <c r="X59" s="92"/>
-      <c r="Y59" s="92"/>
-      <c r="Z59" s="92"/>
-      <c r="AA59" s="92"/>
-      <c r="AB59" s="92"/>
-      <c r="AC59" s="92"/>
-      <c r="AD59" s="92"/>
-      <c r="AE59" s="92"/>
-      <c r="AF59" s="92"/>
-      <c r="AG59" s="92"/>
-      <c r="AH59" s="92"/>
-      <c r="AI59" s="92"/>
+      <c r="A59" s="147"/>
+      <c r="B59" s="147"/>
+      <c r="C59" s="147"/>
+      <c r="D59" s="147"/>
+      <c r="E59" s="147"/>
+      <c r="F59" s="147"/>
+      <c r="G59" s="147"/>
+      <c r="H59" s="147"/>
+      <c r="I59" s="147"/>
+      <c r="J59" s="147"/>
+      <c r="K59" s="147"/>
+      <c r="L59" s="147"/>
+      <c r="M59" s="147"/>
+      <c r="N59" s="147"/>
+      <c r="O59" s="147"/>
+      <c r="P59" s="147"/>
+      <c r="Q59" s="147"/>
+      <c r="R59" s="147"/>
+      <c r="S59" s="147"/>
+      <c r="T59" s="147"/>
+      <c r="U59" s="147"/>
+      <c r="V59" s="147"/>
+      <c r="W59" s="147"/>
+      <c r="X59" s="147"/>
+      <c r="Y59" s="147"/>
+      <c r="Z59" s="147"/>
+      <c r="AA59" s="147"/>
+      <c r="AB59" s="147"/>
+      <c r="AC59" s="147"/>
+      <c r="AD59" s="147"/>
+      <c r="AE59" s="147"/>
+      <c r="AF59" s="147"/>
+      <c r="AG59" s="147"/>
+      <c r="AH59" s="147"/>
+      <c r="AI59" s="147"/>
       <c r="AJ59" s="39"/>
       <c r="AO59" s="38"/>
       <c r="AP59" s="38"/>
@@ -5455,7 +5506,7 @@
       <c r="AS60" s="38"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="1aTPuEU3NhZjJxWnpGrRbE8z33Z8qF+21N+NTPhW09yNT+tGoBaneH6+Ah1jh0fdRbAFhL1OJNKW9GCixmfDGg==" saltValue="Glx0sIOwdUvuMibkfUajtw==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="5BBRMmwV3ZPe4SmOvUFOxncfHHwKnQ3H/M2AENv5ykzgDH+flpWjumNdssrF8ChdtzP2iK58pw+1C1dJeP8Tow==" saltValue="AQfJfyTIPJaUMzb2UsMdjg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0"/>
   <protectedRanges>
     <protectedRange sqref="A2 A5 A7:N7 A8:AI8 A9:I10 J10 A11:E12 F12 AI11 A13:H15 I15" name="Диапазон1"/>
     <protectedRange sqref="A2 A16:Q17 R17:U17 U16:AI17 Q19:AI19 AD18 W18 A18:P19 A20:AI20 C47 S48:V48 D49:R49 Y49:Z49 X48:AC48 AE48:AI49 E47:R47" name="Диапазон2"/>
@@ -5466,6 +5517,176 @@
     <protectedRange sqref="G55:T55 A56:AI59 A55:E55 X52:AI55 U52:U55 V53:W55" name="Диапазон7"/>
   </protectedRanges>
   <mergeCells count="194">
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:N38"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:M40"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="Y35:Z35"/>
+    <mergeCell ref="W35:X35"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="K34:Q34"/>
+    <mergeCell ref="S34:Z34"/>
+    <mergeCell ref="S36:Z36"/>
+    <mergeCell ref="S35:T35"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="W24:X24"/>
+    <mergeCell ref="Y24:Z24"/>
+    <mergeCell ref="W29:X29"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="S28:T28"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="A58:AI59"/>
+    <mergeCell ref="A56:AI57"/>
+    <mergeCell ref="H55:J55"/>
+    <mergeCell ref="K39:Q39"/>
+    <mergeCell ref="S39:Z39"/>
+    <mergeCell ref="X48:Y48"/>
+    <mergeCell ref="Z48:AA48"/>
+    <mergeCell ref="AB48:AC48"/>
+    <mergeCell ref="S47:V47"/>
+    <mergeCell ref="AB47:AC47"/>
+    <mergeCell ref="AE48:AI49"/>
+    <mergeCell ref="Z43:AI44"/>
+    <mergeCell ref="Q43:X45"/>
+    <mergeCell ref="L55:T55"/>
+    <mergeCell ref="B50:L50"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="Q46:X46"/>
+    <mergeCell ref="Z54:AI54"/>
+    <mergeCell ref="Y40:Z40"/>
+    <mergeCell ref="B45:O45"/>
+    <mergeCell ref="Z45:AI45"/>
+    <mergeCell ref="U40:V40"/>
+    <mergeCell ref="X52:Y52"/>
+    <mergeCell ref="Z52:AI53"/>
+    <mergeCell ref="B18:P18"/>
+    <mergeCell ref="J21:M21"/>
+    <mergeCell ref="B19:P19"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="K33:R33"/>
+    <mergeCell ref="S33:Z33"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="Y26:Z26"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="Y29:Z29"/>
+    <mergeCell ref="U28:V28"/>
+    <mergeCell ref="S26:T26"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="W26:X26"/>
+    <mergeCell ref="B30:P30"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="U29:V29"/>
+    <mergeCell ref="R30:T30"/>
+    <mergeCell ref="B32:Q32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="AB19:AC19"/>
+    <mergeCell ref="X19:Y19"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="A2:AI4"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="B7:N7"/>
+    <mergeCell ref="B9:J9"/>
+    <mergeCell ref="Q18:V18"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="R16:T16"/>
+    <mergeCell ref="A5:AI6"/>
+    <mergeCell ref="Z18:AA18"/>
+    <mergeCell ref="AE19:AI20"/>
+    <mergeCell ref="N21:Q21"/>
+    <mergeCell ref="I15:AI15"/>
+    <mergeCell ref="B16:Q16"/>
+    <mergeCell ref="AB18:AC18"/>
+    <mergeCell ref="AE18:AI18"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="Q19:V19"/>
+    <mergeCell ref="O8:AI8"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="Z19:AA19"/>
+    <mergeCell ref="F12:AI12"/>
+    <mergeCell ref="AB21:AE21"/>
+    <mergeCell ref="AF21:AI21"/>
+    <mergeCell ref="S22:T22"/>
+    <mergeCell ref="U22:V22"/>
+    <mergeCell ref="J10:AI10"/>
+    <mergeCell ref="F11:AH11"/>
+    <mergeCell ref="X18:Y18"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="I13:AI14"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="U35:V35"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="A1:AI1"/>
+    <mergeCell ref="S40:T40"/>
+    <mergeCell ref="AB40:AI40"/>
+    <mergeCell ref="B42:P42"/>
+    <mergeCell ref="W40:X40"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="W22:X22"/>
+    <mergeCell ref="Y22:Z22"/>
+    <mergeCell ref="AA22:AB22"/>
+    <mergeCell ref="AC22:AD22"/>
+    <mergeCell ref="AE22:AF22"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AC24:AD24"/>
+    <mergeCell ref="AE24:AF24"/>
+    <mergeCell ref="AG22:AH22"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="W23:X23"/>
+    <mergeCell ref="Y23:Z23"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="K35:Q36"/>
+    <mergeCell ref="AB33:AI33"/>
+    <mergeCell ref="AB34:AI35"/>
+    <mergeCell ref="C39:I39"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C33:I33"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="U37:V37"/>
+    <mergeCell ref="W37:X37"/>
+    <mergeCell ref="Y37:Z37"/>
+    <mergeCell ref="AB37:AI37"/>
+    <mergeCell ref="O37:Q37"/>
+    <mergeCell ref="S37:T37"/>
+    <mergeCell ref="L53:T53"/>
+    <mergeCell ref="H53:J53"/>
+    <mergeCell ref="AE47:AI47"/>
+    <mergeCell ref="S48:V49"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="Z47:AA47"/>
+    <mergeCell ref="X47:Y47"/>
+    <mergeCell ref="B43:O44"/>
+    <mergeCell ref="O40:Q40"/>
     <mergeCell ref="O7:W7"/>
     <mergeCell ref="X7:Y7"/>
     <mergeCell ref="K9:W9"/>
@@ -5490,176 +5711,6 @@
     <mergeCell ref="K26:L26"/>
     <mergeCell ref="U21:Z21"/>
     <mergeCell ref="B20:L20"/>
-    <mergeCell ref="L53:T53"/>
-    <mergeCell ref="H53:J53"/>
-    <mergeCell ref="AE47:AI47"/>
-    <mergeCell ref="S48:V49"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="Z47:AA47"/>
-    <mergeCell ref="X47:Y47"/>
-    <mergeCell ref="B43:O44"/>
-    <mergeCell ref="O40:Q40"/>
-    <mergeCell ref="C35:I35"/>
-    <mergeCell ref="K35:Q36"/>
-    <mergeCell ref="AB33:AI33"/>
-    <mergeCell ref="AB34:AI35"/>
-    <mergeCell ref="C39:I39"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C33:I33"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="C34:I34"/>
-    <mergeCell ref="U37:V37"/>
-    <mergeCell ref="W37:X37"/>
-    <mergeCell ref="Y37:Z37"/>
-    <mergeCell ref="AB37:AI37"/>
-    <mergeCell ref="O37:Q37"/>
-    <mergeCell ref="S37:T37"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="U35:V35"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="A1:AI1"/>
-    <mergeCell ref="S40:T40"/>
-    <mergeCell ref="AB40:AI40"/>
-    <mergeCell ref="B42:P42"/>
-    <mergeCell ref="W40:X40"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="W22:X22"/>
-    <mergeCell ref="Y22:Z22"/>
-    <mergeCell ref="AA22:AB22"/>
-    <mergeCell ref="AC22:AD22"/>
-    <mergeCell ref="AE22:AF22"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AC24:AD24"/>
-    <mergeCell ref="AE24:AF24"/>
-    <mergeCell ref="AG22:AH22"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="W23:X23"/>
-    <mergeCell ref="Y23:Z23"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="Q19:V19"/>
-    <mergeCell ref="O8:AI8"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="Z19:AA19"/>
-    <mergeCell ref="F12:AI12"/>
-    <mergeCell ref="AB21:AE21"/>
-    <mergeCell ref="AF21:AI21"/>
-    <mergeCell ref="S22:T22"/>
-    <mergeCell ref="U22:V22"/>
-    <mergeCell ref="J10:AI10"/>
-    <mergeCell ref="F11:AH11"/>
-    <mergeCell ref="X18:Y18"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="I13:AI14"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="AB19:AC19"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="O22:P22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="A2:AI4"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="B7:N7"/>
-    <mergeCell ref="B9:J9"/>
-    <mergeCell ref="Q18:V18"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="R16:T16"/>
-    <mergeCell ref="A5:AI6"/>
-    <mergeCell ref="Z18:AA18"/>
-    <mergeCell ref="AE19:AI20"/>
-    <mergeCell ref="N21:Q21"/>
-    <mergeCell ref="I15:AI15"/>
-    <mergeCell ref="B16:Q16"/>
-    <mergeCell ref="AB18:AC18"/>
-    <mergeCell ref="AE18:AI18"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="B18:P18"/>
-    <mergeCell ref="J21:M21"/>
-    <mergeCell ref="B19:P19"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="K33:R33"/>
-    <mergeCell ref="S33:Z33"/>
-    <mergeCell ref="O26:P26"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="Y26:Z26"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="Y29:Z29"/>
-    <mergeCell ref="U28:V28"/>
-    <mergeCell ref="S26:T26"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="W26:X26"/>
-    <mergeCell ref="B30:P30"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="U29:V29"/>
-    <mergeCell ref="R30:T30"/>
-    <mergeCell ref="B32:Q32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="A58:AI59"/>
-    <mergeCell ref="A56:AI57"/>
-    <mergeCell ref="H55:J55"/>
-    <mergeCell ref="K39:Q39"/>
-    <mergeCell ref="S39:Z39"/>
-    <mergeCell ref="X48:Y48"/>
-    <mergeCell ref="Z48:AA48"/>
-    <mergeCell ref="AB48:AC48"/>
-    <mergeCell ref="S47:V47"/>
-    <mergeCell ref="AB47:AC47"/>
-    <mergeCell ref="AE48:AI49"/>
-    <mergeCell ref="Z43:AI44"/>
-    <mergeCell ref="Q43:X45"/>
-    <mergeCell ref="L55:T55"/>
-    <mergeCell ref="B50:L50"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="Q46:X46"/>
-    <mergeCell ref="Z54:AI54"/>
-    <mergeCell ref="Y40:Z40"/>
-    <mergeCell ref="B45:O45"/>
-    <mergeCell ref="Z45:AI45"/>
-    <mergeCell ref="U40:V40"/>
-    <mergeCell ref="X52:Y52"/>
-    <mergeCell ref="Z52:AI53"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:N38"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:M40"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="Y35:Z35"/>
-    <mergeCell ref="W35:X35"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="K34:Q34"/>
-    <mergeCell ref="S34:Z34"/>
-    <mergeCell ref="S36:Z36"/>
-    <mergeCell ref="S35:T35"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="W24:X24"/>
-    <mergeCell ref="Y24:Z24"/>
-    <mergeCell ref="W29:X29"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="S28:T28"/>
-    <mergeCell ref="S24:T24"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <dataValidations count="12">
@@ -5679,7 +5730,7 @@
       <formula1>$AP$19:$AP$30</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB18:AC18" xr:uid="{00000000-0002-0000-0000-000005000000}">
-      <formula1>$AQ$19:$AQ$54</formula1>
+      <formula1>$AQ$19:$AQ$55</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S47:V47" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>$AS$19:$AS$21</formula1>
@@ -5697,8 +5748,8 @@
       <formula1>0</formula1>
       <formula2>9</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G22:H22 G24:H24 G26:H26 G28:H28 Y22:Z22 Y24:Z24 Y26:Z26 Y28:Z28 AB47:AC47" xr:uid="{776B72EB-27BC-481F-8B1D-D697A319E1B7}">
-      <formula1>$AQ$19:$AQ$54</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y22:Z22 Y24:Z24 Y26:Z26 Y28:Z28 G22:H22 G24:H24 G26:H26 G28:H28 AB47:AC47" xr:uid="{0C5EA983-1A15-4FA1-90BC-BCF0E25A17AF}">
+      <formula1>$AQ$19:$AQ$55</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.43307086614173229" right="0.15748031496062992" top="0.15748031496062992" bottom="7.874015748031496E-2" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>